<commit_message>
Gantt: 09:00-17:00 with lunch slot, IMHS and Cutting Edge seminars, lectures and journal clubs, week 4 rebuilt
Course hours 09:00-17:00, lunch 12:00-13:00 as its own cell. Mondays 12:00
IMHS Lunch Seminar, Tuesdays 16:00 slot Cutting Edge Immunology Seminar
(weeks 2-4). Week 2: Wed lecture tissue repair I, Thu journal club 1.
Week 3: Tue lecture single-cell transcriptomics, Thu journal club 2.
Week 4: student-organised event removed; Wed writing lecture, poster
production, failure round; Thu poster production, printing deadline 14:00,
recap and Q&A; Fri clean-up, feedback round, poster presentations, Apéro.
Legend and Overview updated. Mirror regenerated.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -22,7 +22,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -90,6 +90,12 @@
     </font>
     <font>
       <name val="Arial"/>
+      <sz val="9"/>
+    </font>
+    <font/>
+    <font>
+      <name val="Arial"/>
+      <color rgb="005A5A5A"/>
       <sz val="9"/>
     </font>
   </fonts>
@@ -279,7 +285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -376,6 +382,13 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -880,7 +893,7 @@
       </c>
       <c r="B14" s="14" t="inlineStr">
         <is>
-          <t>One sheet per week. Eight cells per day: four in the morning, four in the afternoon, one per hour. Rows: fixed layer, one row per group, shared staff row, resources, notes.</t>
+          <t>One sheet per week, course hours 09:00-17:00. Eight cells per day, one per hour: three in the morning, lunch 12:00-13:00, four in the afternoon. Rows: fixed layer, one row per group, shared staff row, resources, notes.</t>
         </is>
       </c>
     </row>
@@ -892,7 +905,7 @@
       </c>
       <c r="B15" s="14" t="inlineStr">
         <is>
-          <t>Lecture slots, facility lecture, cytometer slots, writing day, poster day. Drawn by the teaching staff, thick border, locked. Everything else is flexible.</t>
+          <t>Lecture slots, journal clubs, facility lecture, cytometer slots, the Monday IMHS Lunch Seminar and the Tuesday Cutting Edge Immunology Seminar (16:30-17:30), writing lecture, recap, presentations. Drawn by the teaching staff, thick border, locked. Everything else is flexible.</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1040,7 @@
     <row r="31">
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>[TODO] Poster printing: where, deadline.</t>
+          <t>[TODO] Poster printing: printer. Deadline is Thu 15 Apr 14:00 (poster PDF committed to the group branch).</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1055,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1197,22 +1210,22 @@
       </c>
       <c r="C8" s="23" t="inlineStr">
         <is>
-          <t>Extensions; evening event</t>
+          <t>Extensions</t>
         </is>
       </c>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>Writing day; failure round</t>
+          <t>Writing lecture; poster production; failure round</t>
         </is>
       </c>
       <c r="E8" s="24" t="inlineStr">
         <is>
-          <t>Poster production; feedback</t>
+          <t>Poster production; printing deadline 14:00; recap and Q&amp;A</t>
         </is>
       </c>
       <c r="F8" s="18" t="inlineStr">
         <is>
-          <t>Presentations, prize</t>
+          <t>Clean-up, feedback; poster presentations, prize, Apéro</t>
         </is>
       </c>
     </row>
@@ -1220,6 +1233,13 @@
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Every day in weeks 2 to 4 (Mon-Tue) is half wet lab, half dry lab per group; see the week sheets.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Course hours 09:00-17:00, lunch 12:00-13:00. Weeks 2-4: IMHS Lunch Seminar Mon 12:00-13:00, Cutting Edge Immunology Seminar Tue 16:30-17:30.</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1279,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Week 1: orientation (Thu 18 - Fri 19 March 2027)</t>
+          <t>Week 1: orientation (Thu 18 - Fri 19 March 2027), 09:00-17:00</t>
         </is>
       </c>
     </row>
@@ -1281,25 +1301,25 @@
           <t>Thu 18 Mar</t>
         </is>
       </c>
-      <c r="C3" s="25" t="n"/>
-      <c r="D3" s="25" t="n"/>
-      <c r="E3" s="25" t="n"/>
-      <c r="F3" s="25" t="n"/>
-      <c r="G3" s="25" t="n"/>
-      <c r="H3" s="25" t="n"/>
-      <c r="I3" s="25" t="n"/>
+      <c r="C3" s="32" t="n"/>
+      <c r="D3" s="32" t="n"/>
+      <c r="E3" s="32" t="n"/>
+      <c r="F3" s="32" t="n"/>
+      <c r="G3" s="32" t="n"/>
+      <c r="H3" s="32" t="n"/>
+      <c r="I3" s="33" t="n"/>
       <c r="J3" s="25" t="inlineStr">
         <is>
           <t>Fri 19 Mar</t>
         </is>
       </c>
-      <c r="K3" s="25" t="n"/>
-      <c r="L3" s="25" t="n"/>
-      <c r="M3" s="25" t="n"/>
-      <c r="N3" s="25" t="n"/>
-      <c r="O3" s="25" t="n"/>
-      <c r="P3" s="25" t="n"/>
-      <c r="Q3" s="25" t="n"/>
+      <c r="K3" s="32" t="n"/>
+      <c r="L3" s="32" t="n"/>
+      <c r="M3" s="32" t="n"/>
+      <c r="N3" s="32" t="n"/>
+      <c r="O3" s="32" t="n"/>
+      <c r="P3" s="32" t="n"/>
+      <c r="Q3" s="33" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
@@ -1309,36 +1329,44 @@
       </c>
       <c r="B4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="C4" s="25" t="n"/>
-      <c r="D4" s="25" t="n"/>
-      <c r="E4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="n"/>
+      <c r="D4" s="33" t="n"/>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="G4" s="25" t="n"/>
-      <c r="H4" s="25" t="n"/>
-      <c r="I4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="G4" s="32" t="n"/>
+      <c r="H4" s="32" t="n"/>
+      <c r="I4" s="33" t="n"/>
       <c r="J4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="K4" s="25" t="n"/>
-      <c r="L4" s="25" t="n"/>
-      <c r="M4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="K4" s="32" t="n"/>
+      <c r="L4" s="33" t="n"/>
+      <c r="M4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="N4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="O4" s="25" t="n"/>
-      <c r="P4" s="25" t="n"/>
-      <c r="Q4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="O4" s="32" t="n"/>
+      <c r="P4" s="32" t="n"/>
+      <c r="Q4" s="33" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -1348,82 +1376,82 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="H5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="I5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="K5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="L5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="M5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="N5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="O5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="P5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="Q5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
     </row>
@@ -1439,13 +1467,13 @@
           <t>Welcome, safety briefing, group formation</t>
         </is>
       </c>
-      <c r="C6" s="28" t="n"/>
-      <c r="D6" s="27" t="inlineStr">
-        <is>
-          <t>Lecture: tissue macrophages and nomenclature (recap of Immunology III)</t>
-        </is>
-      </c>
-      <c r="E6" s="28" t="n"/>
+      <c r="C6" s="27" t="inlineStr">
+        <is>
+          <t>Lecture: tissue macrophages and nomenclature</t>
+        </is>
+      </c>
+      <c r="D6" s="28" t="n"/>
+      <c r="E6" s="40" t="n"/>
       <c r="F6" s="27" t="inlineStr">
         <is>
           <t>Lecture: the techniques of this course, one slide per method</t>
@@ -1457,7 +1485,7 @@
       <c r="J6" s="17" t="n"/>
       <c r="K6" s="17" t="n"/>
       <c r="L6" s="17" t="n"/>
-      <c r="M6" s="17" t="n"/>
+      <c r="M6" s="41" t="n"/>
       <c r="N6" s="29" t="inlineStr">
         <is>
           <t>Facility lecture: flow cytometry and FlowJo [TODO: confirm slot with the facility]</t>
@@ -1480,8 +1508,12 @@
         </is>
       </c>
       <c r="C7" s="30" t="n"/>
-      <c r="D7" s="30" t="n"/>
-      <c r="E7" s="28" t="n"/>
+      <c r="D7" s="28" t="n"/>
+      <c r="E7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="F7" s="27" t="inlineStr">
         <is>
           <t>Lecture</t>
@@ -1500,8 +1532,12 @@
         </is>
       </c>
       <c r="K7" s="32" t="n"/>
-      <c r="L7" s="32" t="n"/>
-      <c r="M7" s="33" t="n"/>
+      <c r="L7" s="33" t="n"/>
+      <c r="M7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N7" s="29" t="inlineStr">
         <is>
           <t>Facility lecture</t>
@@ -1528,8 +1564,12 @@
         </is>
       </c>
       <c r="C8" s="30" t="n"/>
-      <c r="D8" s="30" t="n"/>
-      <c r="E8" s="28" t="n"/>
+      <c r="D8" s="28" t="n"/>
+      <c r="E8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="F8" s="27" t="inlineStr">
         <is>
           <t>Lecture</t>
@@ -1548,8 +1588,12 @@
         </is>
       </c>
       <c r="K8" s="32" t="n"/>
-      <c r="L8" s="32" t="n"/>
-      <c r="M8" s="33" t="n"/>
+      <c r="L8" s="33" t="n"/>
+      <c r="M8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N8" s="29" t="inlineStr">
         <is>
           <t>Facility lecture</t>
@@ -1576,8 +1620,12 @@
         </is>
       </c>
       <c r="C9" s="30" t="n"/>
-      <c r="D9" s="30" t="n"/>
-      <c r="E9" s="28" t="n"/>
+      <c r="D9" s="28" t="n"/>
+      <c r="E9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="F9" s="27" t="inlineStr">
         <is>
           <t>Lecture</t>
@@ -1596,8 +1644,12 @@
         </is>
       </c>
       <c r="K9" s="32" t="n"/>
-      <c r="L9" s="32" t="n"/>
-      <c r="M9" s="33" t="n"/>
+      <c r="L9" s="33" t="n"/>
+      <c r="M9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N9" s="29" t="inlineStr">
         <is>
           <t>Facility lecture</t>
@@ -1624,8 +1676,12 @@
         </is>
       </c>
       <c r="C10" s="30" t="n"/>
-      <c r="D10" s="30" t="n"/>
-      <c r="E10" s="28" t="n"/>
+      <c r="D10" s="28" t="n"/>
+      <c r="E10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="F10" s="27" t="inlineStr">
         <is>
           <t>Lecture</t>
@@ -1644,8 +1700,12 @@
         </is>
       </c>
       <c r="K10" s="32" t="n"/>
-      <c r="L10" s="32" t="n"/>
-      <c r="M10" s="33" t="n"/>
+      <c r="L10" s="33" t="n"/>
+      <c r="M10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N10" s="29" t="inlineStr">
         <is>
           <t>Facility lecture</t>
@@ -1668,7 +1728,7 @@
       </c>
       <c r="B11" s="34" t="inlineStr">
         <is>
-          <t>Rooms, safety officer, group list. Supervisors sit with their group from 14:30.</t>
+          <t>Rooms, safety officer, group list. Supervisors sit with their group from 14:00.</t>
         </is>
       </c>
       <c r="C11" s="32" t="n"/>
@@ -1747,41 +1807,40 @@
       <c r="Q13" s="35" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="35">
-    <mergeCell ref="B9:E9"/>
+  <mergeCells count="34">
     <mergeCell ref="G10:I10"/>
+    <mergeCell ref="C6:D6"/>
     <mergeCell ref="N7:O7"/>
+    <mergeCell ref="B8:D8"/>
     <mergeCell ref="P10:Q10"/>
     <mergeCell ref="B3:I3"/>
+    <mergeCell ref="J4:L4"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="B12:I12"/>
-    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="B10:D10"/>
     <mergeCell ref="P9:Q9"/>
-    <mergeCell ref="B4:E4"/>
+    <mergeCell ref="J7:L7"/>
     <mergeCell ref="B11:I11"/>
     <mergeCell ref="F4:I4"/>
-    <mergeCell ref="J8:M8"/>
     <mergeCell ref="P8:Q8"/>
     <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="B7:E7"/>
+    <mergeCell ref="B9:D9"/>
     <mergeCell ref="N8:O8"/>
-    <mergeCell ref="J10:M10"/>
     <mergeCell ref="P7:Q7"/>
-    <mergeCell ref="J9:M9"/>
     <mergeCell ref="J11:Q11"/>
+    <mergeCell ref="B4:D4"/>
     <mergeCell ref="N10:O10"/>
     <mergeCell ref="A2:Q2"/>
     <mergeCell ref="G9:I9"/>
-    <mergeCell ref="J7:M7"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="B7:D7"/>
     <mergeCell ref="N9:O9"/>
-    <mergeCell ref="B6:C6"/>
-    <mergeCell ref="B8:E8"/>
     <mergeCell ref="J12:Q12"/>
+    <mergeCell ref="J10:L10"/>
     <mergeCell ref="J3:Q3"/>
     <mergeCell ref="N6:O6"/>
-    <mergeCell ref="J4:M4"/>
     <mergeCell ref="G8:I8"/>
-    <mergeCell ref="B10:E10"/>
+    <mergeCell ref="J9:L9"/>
     <mergeCell ref="G7:I7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1857,49 +1916,49 @@
           <t>Mon 22 Mar</t>
         </is>
       </c>
-      <c r="C3" s="25" t="n"/>
-      <c r="D3" s="25" t="n"/>
-      <c r="E3" s="25" t="n"/>
-      <c r="F3" s="25" t="n"/>
-      <c r="G3" s="25" t="n"/>
-      <c r="H3" s="25" t="n"/>
-      <c r="I3" s="25" t="n"/>
+      <c r="C3" s="32" t="n"/>
+      <c r="D3" s="32" t="n"/>
+      <c r="E3" s="32" t="n"/>
+      <c r="F3" s="32" t="n"/>
+      <c r="G3" s="32" t="n"/>
+      <c r="H3" s="32" t="n"/>
+      <c r="I3" s="33" t="n"/>
       <c r="J3" s="25" t="inlineStr">
         <is>
           <t>Tue 23 Mar</t>
         </is>
       </c>
-      <c r="K3" s="25" t="n"/>
-      <c r="L3" s="25" t="n"/>
-      <c r="M3" s="25" t="n"/>
-      <c r="N3" s="25" t="n"/>
-      <c r="O3" s="25" t="n"/>
-      <c r="P3" s="25" t="n"/>
-      <c r="Q3" s="25" t="n"/>
+      <c r="K3" s="32" t="n"/>
+      <c r="L3" s="32" t="n"/>
+      <c r="M3" s="32" t="n"/>
+      <c r="N3" s="32" t="n"/>
+      <c r="O3" s="32" t="n"/>
+      <c r="P3" s="32" t="n"/>
+      <c r="Q3" s="33" t="n"/>
       <c r="R3" s="25" t="inlineStr">
         <is>
           <t>Wed 24 Mar</t>
         </is>
       </c>
-      <c r="S3" s="25" t="n"/>
-      <c r="T3" s="25" t="n"/>
-      <c r="U3" s="25" t="n"/>
-      <c r="V3" s="25" t="n"/>
-      <c r="W3" s="25" t="n"/>
-      <c r="X3" s="25" t="n"/>
-      <c r="Y3" s="25" t="n"/>
+      <c r="S3" s="32" t="n"/>
+      <c r="T3" s="32" t="n"/>
+      <c r="U3" s="32" t="n"/>
+      <c r="V3" s="32" t="n"/>
+      <c r="W3" s="32" t="n"/>
+      <c r="X3" s="32" t="n"/>
+      <c r="Y3" s="33" t="n"/>
       <c r="Z3" s="25" t="inlineStr">
         <is>
           <t>Thu 25 Mar</t>
         </is>
       </c>
-      <c r="AA3" s="25" t="n"/>
-      <c r="AB3" s="25" t="n"/>
-      <c r="AC3" s="25" t="n"/>
-      <c r="AD3" s="25" t="n"/>
-      <c r="AE3" s="25" t="n"/>
-      <c r="AF3" s="25" t="n"/>
-      <c r="AG3" s="25" t="n"/>
+      <c r="AA3" s="32" t="n"/>
+      <c r="AB3" s="32" t="n"/>
+      <c r="AC3" s="32" t="n"/>
+      <c r="AD3" s="32" t="n"/>
+      <c r="AE3" s="32" t="n"/>
+      <c r="AF3" s="32" t="n"/>
+      <c r="AG3" s="33" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
@@ -1909,68 +1968,84 @@
       </c>
       <c r="B4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="C4" s="25" t="n"/>
-      <c r="D4" s="25" t="n"/>
-      <c r="E4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="n"/>
+      <c r="D4" s="33" t="n"/>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="G4" s="25" t="n"/>
-      <c r="H4" s="25" t="n"/>
-      <c r="I4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="G4" s="32" t="n"/>
+      <c r="H4" s="32" t="n"/>
+      <c r="I4" s="33" t="n"/>
       <c r="J4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="K4" s="25" t="n"/>
-      <c r="L4" s="25" t="n"/>
-      <c r="M4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="K4" s="32" t="n"/>
+      <c r="L4" s="33" t="n"/>
+      <c r="M4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="N4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="O4" s="25" t="n"/>
-      <c r="P4" s="25" t="n"/>
-      <c r="Q4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="O4" s="32" t="n"/>
+      <c r="P4" s="32" t="n"/>
+      <c r="Q4" s="33" t="n"/>
       <c r="R4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="S4" s="25" t="n"/>
-      <c r="T4" s="25" t="n"/>
-      <c r="U4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="S4" s="32" t="n"/>
+      <c r="T4" s="33" t="n"/>
+      <c r="U4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="V4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="W4" s="25" t="n"/>
-      <c r="X4" s="25" t="n"/>
-      <c r="Y4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="W4" s="32" t="n"/>
+      <c r="X4" s="32" t="n"/>
+      <c r="Y4" s="33" t="n"/>
       <c r="Z4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="AA4" s="25" t="n"/>
-      <c r="AB4" s="25" t="n"/>
-      <c r="AC4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="AA4" s="32" t="n"/>
+      <c r="AB4" s="33" t="n"/>
+      <c r="AC4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="AD4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="AE4" s="25" t="n"/>
-      <c r="AF4" s="25" t="n"/>
-      <c r="AG4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="AE4" s="32" t="n"/>
+      <c r="AF4" s="32" t="n"/>
+      <c r="AG4" s="33" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -1980,162 +2055,162 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="H5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="I5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="K5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="L5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="M5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="N5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="O5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="P5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="Q5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="R5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="S5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="T5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="U5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="V5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="W5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="X5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="Y5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="Z5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="AA5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="AB5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="AC5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="AD5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="AE5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="AF5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="AG5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2224,11 @@
       <c r="B6" s="17" t="n"/>
       <c r="C6" s="17" t="n"/>
       <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F6" s="17" t="n"/>
       <c r="G6" s="17" t="n"/>
       <c r="H6" s="17" t="n"/>
@@ -2157,23 +2236,35 @@
       <c r="J6" s="17" t="n"/>
       <c r="K6" s="17" t="n"/>
       <c r="L6" s="17" t="n"/>
-      <c r="M6" s="17" t="n"/>
+      <c r="M6" s="41" t="n"/>
       <c r="N6" s="17" t="n"/>
       <c r="O6" s="17" t="n"/>
       <c r="P6" s="17" t="n"/>
-      <c r="Q6" s="17" t="n"/>
-      <c r="R6" s="17" t="n"/>
+      <c r="Q6" s="27" t="inlineStr">
+        <is>
+          <t>Cutting Edge Immunology Seminar 16:30-17:30</t>
+        </is>
+      </c>
+      <c r="R6" s="27" t="inlineStr">
+        <is>
+          <t>Lecture: tissue repair I, macrophages in injury and repair</t>
+        </is>
+      </c>
       <c r="S6" s="17" t="n"/>
       <c r="T6" s="17" t="n"/>
-      <c r="U6" s="17" t="n"/>
+      <c r="U6" s="41" t="n"/>
       <c r="V6" s="17" t="n"/>
       <c r="W6" s="17" t="n"/>
       <c r="X6" s="17" t="n"/>
       <c r="Y6" s="17" t="n"/>
-      <c r="Z6" s="17" t="n"/>
+      <c r="Z6" s="27" t="inlineStr">
+        <is>
+          <t>Journal club 1: the M1/M2 nomenclature revision [TODO: paper]; one group presents, all read</t>
+        </is>
+      </c>
       <c r="AA6" s="17" t="n"/>
       <c r="AB6" s="17" t="n"/>
-      <c r="AC6" s="17" t="n"/>
+      <c r="AC6" s="41" t="n"/>
       <c r="AD6" s="17" t="n"/>
       <c r="AE6" s="17" t="n"/>
       <c r="AF6" s="17" t="n"/>
@@ -2196,8 +2287,12 @@
         </is>
       </c>
       <c r="C7" s="32" t="n"/>
-      <c r="D7" s="32" t="n"/>
-      <c r="E7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
           <t>Dry lab: analysis templates on example data (ELISA, Griess)</t>
@@ -2212,24 +2307,40 @@
         </is>
       </c>
       <c r="K7" s="32" t="n"/>
-      <c r="L7" s="32" t="n"/>
-      <c r="M7" s="33" t="n"/>
+      <c r="L7" s="33" t="n"/>
+      <c r="M7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N7" s="31" t="inlineStr">
         <is>
           <t>Dry lab: FlowJo on example data. Poster: draft the introduction</t>
         </is>
       </c>
       <c r="O7" s="32" t="n"/>
-      <c r="P7" s="32" t="n"/>
-      <c r="Q7" s="33" t="n"/>
-      <c r="R7" s="36" t="inlineStr">
+      <c r="P7" s="33" t="n"/>
+      <c r="Q7" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
+      <c r="R7" s="27" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="S7" s="36" t="inlineStr">
         <is>
           <t>P02 Count (T2), scrape, split; seed growth-curve wells</t>
         </is>
       </c>
-      <c r="S7" s="32" t="n"/>
-      <c r="T7" s="32" t="n"/>
-      <c r="U7" s="33" t="n"/>
+      <c r="T7" s="33" t="n"/>
+      <c r="U7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="V7" s="31" t="inlineStr">
         <is>
           <t>Dry lab: growth curve and doubling time from your counts. Poster: why does this matter (significance)</t>
@@ -2238,14 +2349,22 @@
       <c r="W7" s="32" t="n"/>
       <c r="X7" s="32" t="n"/>
       <c r="Y7" s="33" t="n"/>
-      <c r="Z7" s="36" t="inlineStr">
+      <c r="Z7" s="27" t="inlineStr">
+        <is>
+          <t>Journal club</t>
+        </is>
+      </c>
+      <c r="AA7" s="36" t="inlineStr">
         <is>
           <t>P01 Count (T3). P03 Freeze your own vials. Clean-up: nothing stays in culture over the break</t>
         </is>
       </c>
-      <c r="AA7" s="32" t="n"/>
-      <c r="AB7" s="32" t="n"/>
-      <c r="AC7" s="33" t="n"/>
+      <c r="AB7" s="33" t="n"/>
+      <c r="AC7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AD7" s="31" t="inlineStr">
         <is>
           <t>Dry lab: scRNA-seq part 1, load the preprocessed object, QC figure</t>
@@ -2272,8 +2391,12 @@
         </is>
       </c>
       <c r="C8" s="32" t="n"/>
-      <c r="D8" s="32" t="n"/>
-      <c r="E8" s="33" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F8" s="31" t="inlineStr">
         <is>
           <t>Dry lab: analysis templates on example data (ELISA, Griess)</t>
@@ -2288,24 +2411,40 @@
         </is>
       </c>
       <c r="K8" s="32" t="n"/>
-      <c r="L8" s="32" t="n"/>
-      <c r="M8" s="33" t="n"/>
+      <c r="L8" s="33" t="n"/>
+      <c r="M8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N8" s="31" t="inlineStr">
         <is>
           <t>Dry lab: FlowJo on example data. Poster: draft the introduction</t>
         </is>
       </c>
       <c r="O8" s="32" t="n"/>
-      <c r="P8" s="32" t="n"/>
-      <c r="Q8" s="33" t="n"/>
-      <c r="R8" s="36" t="inlineStr">
+      <c r="P8" s="33" t="n"/>
+      <c r="Q8" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
+      <c r="R8" s="27" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="S8" s="36" t="inlineStr">
         <is>
           <t>P02 Count (T2), scrape, split; seed growth-curve wells</t>
         </is>
       </c>
-      <c r="S8" s="32" t="n"/>
-      <c r="T8" s="32" t="n"/>
-      <c r="U8" s="33" t="n"/>
+      <c r="T8" s="33" t="n"/>
+      <c r="U8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="V8" s="31" t="inlineStr">
         <is>
           <t>Dry lab: growth curve and doubling time from your counts. Poster: why does this matter (significance)</t>
@@ -2314,14 +2453,22 @@
       <c r="W8" s="32" t="n"/>
       <c r="X8" s="32" t="n"/>
       <c r="Y8" s="33" t="n"/>
-      <c r="Z8" s="36" t="inlineStr">
+      <c r="Z8" s="27" t="inlineStr">
+        <is>
+          <t>Journal club</t>
+        </is>
+      </c>
+      <c r="AA8" s="36" t="inlineStr">
         <is>
           <t>P01 Count (T3). P03 Freeze your own vials. Clean-up: nothing stays in culture over the break</t>
         </is>
       </c>
-      <c r="AA8" s="32" t="n"/>
-      <c r="AB8" s="32" t="n"/>
-      <c r="AC8" s="33" t="n"/>
+      <c r="AB8" s="33" t="n"/>
+      <c r="AC8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AD8" s="31" t="inlineStr">
         <is>
           <t>Dry lab: scRNA-seq part 1, load the preprocessed object, QC figure</t>
@@ -2348,8 +2495,12 @@
         </is>
       </c>
       <c r="C9" s="32" t="n"/>
-      <c r="D9" s="32" t="n"/>
-      <c r="E9" s="33" t="n"/>
+      <c r="D9" s="33" t="n"/>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F9" s="36" t="inlineStr">
         <is>
           <t>P01 Thaw RAW 264.7, count (T0), seed the flask</t>
@@ -2364,24 +2515,40 @@
         </is>
       </c>
       <c r="K9" s="32" t="n"/>
-      <c r="L9" s="32" t="n"/>
-      <c r="M9" s="33" t="n"/>
+      <c r="L9" s="33" t="n"/>
+      <c r="M9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N9" s="36" t="inlineStr">
         <is>
           <t>P01 Inspect, count (T1), medium change</t>
         </is>
       </c>
       <c r="O9" s="32" t="n"/>
-      <c r="P9" s="32" t="n"/>
-      <c r="Q9" s="33" t="n"/>
-      <c r="R9" s="31" t="inlineStr">
+      <c r="P9" s="33" t="n"/>
+      <c r="Q9" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
+      <c r="R9" s="27" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="S9" s="31" t="inlineStr">
         <is>
           <t>Dry lab: growth curve and doubling time from your counts. Poster: why does this matter (significance)</t>
         </is>
       </c>
-      <c r="S9" s="32" t="n"/>
-      <c r="T9" s="32" t="n"/>
-      <c r="U9" s="33" t="n"/>
+      <c r="T9" s="33" t="n"/>
+      <c r="U9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="V9" s="36" t="inlineStr">
         <is>
           <t>P02 Count (T2), scrape, split; seed growth-curve wells</t>
@@ -2390,14 +2557,22 @@
       <c r="W9" s="32" t="n"/>
       <c r="X9" s="32" t="n"/>
       <c r="Y9" s="33" t="n"/>
-      <c r="Z9" s="31" t="inlineStr">
+      <c r="Z9" s="27" t="inlineStr">
+        <is>
+          <t>Journal club</t>
+        </is>
+      </c>
+      <c r="AA9" s="31" t="inlineStr">
         <is>
           <t>Dry lab: scRNA-seq part 1, load the preprocessed object, QC figure</t>
         </is>
       </c>
-      <c r="AA9" s="32" t="n"/>
-      <c r="AB9" s="32" t="n"/>
-      <c r="AC9" s="33" t="n"/>
+      <c r="AB9" s="33" t="n"/>
+      <c r="AC9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AD9" s="36" t="inlineStr">
         <is>
           <t>P01 Count (T3). P03 Freeze your own vials. Clean-up: nothing stays in culture over the break</t>
@@ -2424,8 +2599,12 @@
         </is>
       </c>
       <c r="C10" s="32" t="n"/>
-      <c r="D10" s="32" t="n"/>
-      <c r="E10" s="33" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F10" s="36" t="inlineStr">
         <is>
           <t>P01 Thaw RAW 264.7, count (T0), seed the flask</t>
@@ -2440,24 +2619,40 @@
         </is>
       </c>
       <c r="K10" s="32" t="n"/>
-      <c r="L10" s="32" t="n"/>
-      <c r="M10" s="33" t="n"/>
+      <c r="L10" s="33" t="n"/>
+      <c r="M10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N10" s="36" t="inlineStr">
         <is>
           <t>P01 Inspect, count (T1), medium change</t>
         </is>
       </c>
       <c r="O10" s="32" t="n"/>
-      <c r="P10" s="32" t="n"/>
-      <c r="Q10" s="33" t="n"/>
-      <c r="R10" s="31" t="inlineStr">
+      <c r="P10" s="33" t="n"/>
+      <c r="Q10" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
+      <c r="R10" s="27" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="S10" s="31" t="inlineStr">
         <is>
           <t>Dry lab: growth curve and doubling time from your counts. Poster: why does this matter (significance)</t>
         </is>
       </c>
-      <c r="S10" s="32" t="n"/>
-      <c r="T10" s="32" t="n"/>
-      <c r="U10" s="33" t="n"/>
+      <c r="T10" s="33" t="n"/>
+      <c r="U10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="V10" s="36" t="inlineStr">
         <is>
           <t>P02 Count (T2), scrape, split; seed growth-curve wells</t>
@@ -2466,14 +2661,22 @@
       <c r="W10" s="32" t="n"/>
       <c r="X10" s="32" t="n"/>
       <c r="Y10" s="33" t="n"/>
-      <c r="Z10" s="31" t="inlineStr">
+      <c r="Z10" s="27" t="inlineStr">
+        <is>
+          <t>Journal club</t>
+        </is>
+      </c>
+      <c r="AA10" s="31" t="inlineStr">
         <is>
           <t>Dry lab: scRNA-seq part 1, load the preprocessed object, QC figure</t>
         </is>
       </c>
-      <c r="AA10" s="32" t="n"/>
-      <c r="AB10" s="32" t="n"/>
-      <c r="AC10" s="33" t="n"/>
+      <c r="AB10" s="33" t="n"/>
+      <c r="AC10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AD10" s="36" t="inlineStr">
         <is>
           <t>P01 Count (T3). P03 Freeze your own vials. Clean-up: nothing stays in culture over the break</t>
@@ -2496,7 +2699,7 @@
       </c>
       <c r="B11" s="34" t="inlineStr">
         <is>
-          <t>Medium warmed, one vial per group at 08:30 and 13:30. Supervisor at the hood with the group for the thaw.</t>
+          <t>Medium warmed, one vial per group at 09:00 and 13:00. Supervisor at the hood with the group for the thaw.</t>
         </is>
       </c>
       <c r="C11" s="32" t="n"/>
@@ -2607,7 +2810,7 @@
       </c>
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>Exp 1 is a real experiment: four counts give a growth curve and a doubling time against the published value; viability of your own vial on Mon 5 Apr is the second readout. Easter break Fri 26 Mar to Sun 4 Apr: no course, no cultures.</t>
+          <t>Exp 1 is a real experiment: four counts give a growth curve and a doubling time against the published value; viability of your own vial on Mon 5 Apr is the second readout. Easter break Fri 26 Mar to Sun 4 Apr: no course, no cultures. Mondays 12:00-13:00: IMHS Lunch Seminar. Tuesdays: Cutting Edge Immunology Seminar runs 16:30-17:30.</t>
         </is>
       </c>
       <c r="C13" s="32" t="n"/>
@@ -2645,60 +2848,60 @@
   </sheetData>
   <mergeCells count="55">
     <mergeCell ref="A1:AG1"/>
-    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="F9:I9"/>
+    <mergeCell ref="R11:Y11"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="AD4:AG4"/>
+    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="Z3:AG3"/>
+    <mergeCell ref="Z12:AG12"/>
+    <mergeCell ref="AA7:AB7"/>
+    <mergeCell ref="V8:Y8"/>
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="S10:T10"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="AD9:AF9"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="R3:Y3"/>
+    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="AD8:AF8"/>
+    <mergeCell ref="J12:Q12"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="J9:L9"/>
     <mergeCell ref="AD10:AF10"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="N9:Q9"/>
-    <mergeCell ref="R11:Y11"/>
-    <mergeCell ref="Z4:AC4"/>
+    <mergeCell ref="B8:D8"/>
     <mergeCell ref="Z11:AG11"/>
     <mergeCell ref="B3:I3"/>
     <mergeCell ref="V7:Y7"/>
-    <mergeCell ref="Z10:AC10"/>
+    <mergeCell ref="N8:P8"/>
     <mergeCell ref="B12:I12"/>
-    <mergeCell ref="R9:U9"/>
-    <mergeCell ref="AD4:AG4"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="Z9:AC9"/>
-    <mergeCell ref="R8:U8"/>
-    <mergeCell ref="B11:I11"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="J8:M8"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="N10:P10"/>
     <mergeCell ref="A2:AG2"/>
     <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="N7:Q7"/>
-    <mergeCell ref="R10:U10"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="Z4:AB4"/>
     <mergeCell ref="AD7:AF7"/>
-    <mergeCell ref="Z3:AG3"/>
-    <mergeCell ref="J10:M10"/>
     <mergeCell ref="R12:Y12"/>
-    <mergeCell ref="Z12:AG12"/>
-    <mergeCell ref="R4:U4"/>
-    <mergeCell ref="V8:Y8"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="J9:M9"/>
     <mergeCell ref="V4:Y4"/>
     <mergeCell ref="J11:Q11"/>
-    <mergeCell ref="R7:U7"/>
-    <mergeCell ref="AD9:AF9"/>
+    <mergeCell ref="B13:AG13"/>
     <mergeCell ref="V10:Y10"/>
-    <mergeCell ref="B13:AG13"/>
-    <mergeCell ref="R3:Y3"/>
-    <mergeCell ref="Z7:AC7"/>
-    <mergeCell ref="AD8:AF8"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="B8:E8"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="N7:P7"/>
     <mergeCell ref="V9:Y9"/>
-    <mergeCell ref="N8:Q8"/>
-    <mergeCell ref="J12:Q12"/>
     <mergeCell ref="J3:Q3"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="J4:M4"/>
-    <mergeCell ref="Z8:AC8"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="N10:Q10"/>
+    <mergeCell ref="AA8:AB8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2781,61 +2984,61 @@
           <t>Mon 5 Apr</t>
         </is>
       </c>
-      <c r="C3" s="25" t="n"/>
-      <c r="D3" s="25" t="n"/>
-      <c r="E3" s="25" t="n"/>
-      <c r="F3" s="25" t="n"/>
-      <c r="G3" s="25" t="n"/>
-      <c r="H3" s="25" t="n"/>
-      <c r="I3" s="25" t="n"/>
+      <c r="C3" s="32" t="n"/>
+      <c r="D3" s="32" t="n"/>
+      <c r="E3" s="32" t="n"/>
+      <c r="F3" s="32" t="n"/>
+      <c r="G3" s="32" t="n"/>
+      <c r="H3" s="32" t="n"/>
+      <c r="I3" s="33" t="n"/>
       <c r="J3" s="25" t="inlineStr">
         <is>
           <t>Tue 6 Apr</t>
         </is>
       </c>
-      <c r="K3" s="25" t="n"/>
-      <c r="L3" s="25" t="n"/>
-      <c r="M3" s="25" t="n"/>
-      <c r="N3" s="25" t="n"/>
-      <c r="O3" s="25" t="n"/>
-      <c r="P3" s="25" t="n"/>
-      <c r="Q3" s="25" t="n"/>
+      <c r="K3" s="32" t="n"/>
+      <c r="L3" s="32" t="n"/>
+      <c r="M3" s="32" t="n"/>
+      <c r="N3" s="32" t="n"/>
+      <c r="O3" s="32" t="n"/>
+      <c r="P3" s="32" t="n"/>
+      <c r="Q3" s="33" t="n"/>
       <c r="R3" s="25" t="inlineStr">
         <is>
           <t>Wed 7 Apr</t>
         </is>
       </c>
-      <c r="S3" s="25" t="n"/>
-      <c r="T3" s="25" t="n"/>
-      <c r="U3" s="25" t="n"/>
-      <c r="V3" s="25" t="n"/>
-      <c r="W3" s="25" t="n"/>
-      <c r="X3" s="25" t="n"/>
-      <c r="Y3" s="25" t="n"/>
+      <c r="S3" s="32" t="n"/>
+      <c r="T3" s="32" t="n"/>
+      <c r="U3" s="32" t="n"/>
+      <c r="V3" s="32" t="n"/>
+      <c r="W3" s="32" t="n"/>
+      <c r="X3" s="32" t="n"/>
+      <c r="Y3" s="33" t="n"/>
       <c r="Z3" s="25" t="inlineStr">
         <is>
           <t>Thu 8 Apr</t>
         </is>
       </c>
-      <c r="AA3" s="25" t="n"/>
-      <c r="AB3" s="25" t="n"/>
-      <c r="AC3" s="25" t="n"/>
-      <c r="AD3" s="25" t="n"/>
-      <c r="AE3" s="25" t="n"/>
-      <c r="AF3" s="25" t="n"/>
-      <c r="AG3" s="25" t="n"/>
+      <c r="AA3" s="32" t="n"/>
+      <c r="AB3" s="32" t="n"/>
+      <c r="AC3" s="32" t="n"/>
+      <c r="AD3" s="32" t="n"/>
+      <c r="AE3" s="32" t="n"/>
+      <c r="AF3" s="32" t="n"/>
+      <c r="AG3" s="33" t="n"/>
       <c r="AH3" s="25" t="inlineStr">
         <is>
           <t>Fri 9 Apr</t>
         </is>
       </c>
-      <c r="AI3" s="25" t="n"/>
-      <c r="AJ3" s="25" t="n"/>
-      <c r="AK3" s="25" t="n"/>
-      <c r="AL3" s="25" t="n"/>
-      <c r="AM3" s="25" t="n"/>
-      <c r="AN3" s="25" t="n"/>
-      <c r="AO3" s="25" t="n"/>
+      <c r="AI3" s="32" t="n"/>
+      <c r="AJ3" s="32" t="n"/>
+      <c r="AK3" s="32" t="n"/>
+      <c r="AL3" s="32" t="n"/>
+      <c r="AM3" s="32" t="n"/>
+      <c r="AN3" s="32" t="n"/>
+      <c r="AO3" s="33" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
@@ -2845,84 +3048,104 @@
       </c>
       <c r="B4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="C4" s="25" t="n"/>
-      <c r="D4" s="25" t="n"/>
-      <c r="E4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="n"/>
+      <c r="D4" s="33" t="n"/>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="G4" s="25" t="n"/>
-      <c r="H4" s="25" t="n"/>
-      <c r="I4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="G4" s="32" t="n"/>
+      <c r="H4" s="32" t="n"/>
+      <c r="I4" s="33" t="n"/>
       <c r="J4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="K4" s="25" t="n"/>
-      <c r="L4" s="25" t="n"/>
-      <c r="M4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="K4" s="32" t="n"/>
+      <c r="L4" s="33" t="n"/>
+      <c r="M4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="N4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="O4" s="25" t="n"/>
-      <c r="P4" s="25" t="n"/>
-      <c r="Q4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="O4" s="32" t="n"/>
+      <c r="P4" s="32" t="n"/>
+      <c r="Q4" s="33" t="n"/>
       <c r="R4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="S4" s="25" t="n"/>
-      <c r="T4" s="25" t="n"/>
-      <c r="U4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="S4" s="32" t="n"/>
+      <c r="T4" s="33" t="n"/>
+      <c r="U4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="V4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="W4" s="25" t="n"/>
-      <c r="X4" s="25" t="n"/>
-      <c r="Y4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="W4" s="32" t="n"/>
+      <c r="X4" s="32" t="n"/>
+      <c r="Y4" s="33" t="n"/>
       <c r="Z4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="AA4" s="25" t="n"/>
-      <c r="AB4" s="25" t="n"/>
-      <c r="AC4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="AA4" s="32" t="n"/>
+      <c r="AB4" s="33" t="n"/>
+      <c r="AC4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="AD4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="AE4" s="25" t="n"/>
-      <c r="AF4" s="25" t="n"/>
-      <c r="AG4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="AE4" s="32" t="n"/>
+      <c r="AF4" s="32" t="n"/>
+      <c r="AG4" s="33" t="n"/>
       <c r="AH4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="AI4" s="25" t="n"/>
-      <c r="AJ4" s="25" t="n"/>
-      <c r="AK4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="AI4" s="32" t="n"/>
+      <c r="AJ4" s="33" t="n"/>
+      <c r="AK4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="AL4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="AM4" s="25" t="n"/>
-      <c r="AN4" s="25" t="n"/>
-      <c r="AO4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="AM4" s="32" t="n"/>
+      <c r="AN4" s="32" t="n"/>
+      <c r="AO4" s="33" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -2932,202 +3155,202 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="H5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="I5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="K5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="L5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="M5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="N5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="O5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="P5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="Q5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="R5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="S5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="T5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="U5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="V5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="W5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="X5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="Y5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="Z5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="AA5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="AB5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="AC5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="AD5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="AE5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="AF5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="AG5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="AH5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="AI5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="AJ5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="AK5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="AL5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="AM5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="AN5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="AO5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
     </row>
@@ -3141,19 +3364,31 @@
       <c r="B6" s="17" t="n"/>
       <c r="C6" s="17" t="n"/>
       <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F6" s="17" t="n"/>
       <c r="G6" s="17" t="n"/>
       <c r="H6" s="17" t="n"/>
       <c r="I6" s="17" t="n"/>
-      <c r="J6" s="17" t="n"/>
+      <c r="J6" s="27" t="inlineStr">
+        <is>
+          <t>Lecture: single-cell transcriptomics for immunologists, what a signature score means</t>
+        </is>
+      </c>
       <c r="K6" s="17" t="n"/>
       <c r="L6" s="17" t="n"/>
-      <c r="M6" s="17" t="n"/>
+      <c r="M6" s="41" t="n"/>
       <c r="N6" s="17" t="n"/>
       <c r="O6" s="17" t="n"/>
       <c r="P6" s="17" t="n"/>
-      <c r="Q6" s="17" t="n"/>
+      <c r="Q6" s="27" t="inlineStr">
+        <is>
+          <t>Cutting Edge Immunology Seminar 16:30-17:30</t>
+        </is>
+      </c>
       <c r="R6" s="17" t="n"/>
       <c r="S6" s="17" t="n"/>
       <c r="T6" s="29" t="inlineStr">
@@ -3170,10 +3405,14 @@
         </is>
       </c>
       <c r="Y6" s="28" t="n"/>
-      <c r="Z6" s="17" t="n"/>
+      <c r="Z6" s="27" t="inlineStr">
+        <is>
+          <t>Journal club 2: the peritoneal injury single-cell paper behind GSE186658 [TODO: paper]; one group presents, all read</t>
+        </is>
+      </c>
       <c r="AA6" s="17" t="n"/>
       <c r="AB6" s="17" t="n"/>
-      <c r="AC6" s="17" t="n"/>
+      <c r="AC6" s="41" t="n"/>
       <c r="AD6" s="17" t="n"/>
       <c r="AE6" s="17" t="n"/>
       <c r="AF6" s="17" t="n"/>
@@ -3181,7 +3420,7 @@
       <c r="AH6" s="17" t="n"/>
       <c r="AI6" s="17" t="n"/>
       <c r="AJ6" s="17" t="n"/>
-      <c r="AK6" s="17" t="n"/>
+      <c r="AK6" s="41" t="n"/>
       <c r="AL6" s="17" t="n"/>
       <c r="AM6" s="17" t="n"/>
       <c r="AN6" s="17" t="n"/>
@@ -3204,8 +3443,12 @@
         </is>
       </c>
       <c r="C7" s="32" t="n"/>
-      <c r="D7" s="32" t="n"/>
-      <c r="E7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F7" s="37" t="inlineStr">
         <is>
           <t>P01 Thaw your own vial (viability = Exp 1 readout). P02 Seed Exp 2 plates from the staff culture</t>
@@ -3214,30 +3457,46 @@
       <c r="G7" s="32" t="n"/>
       <c r="H7" s="32" t="n"/>
       <c r="I7" s="33" t="n"/>
-      <c r="J7" s="31" t="inlineStr">
+      <c r="J7" s="27" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="K7" s="31" t="inlineStr">
         <is>
           <t>Dry lab: scRNA-seq part 3, score the tissue macrophages. Poster: methods</t>
         </is>
       </c>
-      <c r="K7" s="32" t="n"/>
-      <c r="L7" s="32" t="n"/>
-      <c r="M7" s="33" t="n"/>
+      <c r="L7" s="33" t="n"/>
+      <c r="M7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N7" s="37" t="inlineStr">
         <is>
           <t>P04 Polarize: M(-), M(IFNg), M(IL-4), M(IFNg+LPS), 24 h</t>
         </is>
       </c>
       <c r="O7" s="32" t="n"/>
-      <c r="P7" s="32" t="n"/>
-      <c r="Q7" s="33" t="n"/>
+      <c r="P7" s="33" t="n"/>
+      <c r="Q7" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
       <c r="R7" s="31" t="inlineStr">
         <is>
           <t>Dry lab: FlowJo gating of your own data, export statistics</t>
         </is>
       </c>
       <c r="S7" s="32" t="n"/>
-      <c r="T7" s="32" t="n"/>
-      <c r="U7" s="33" t="n"/>
+      <c r="T7" s="33" t="n"/>
+      <c r="U7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="V7" s="37" t="inlineStr">
         <is>
           <t>P04 Wash. P05 Challenge: LPS + your axis, 24 h. P08 Stain the unchallenged wells, acquire in the facility slot</t>
@@ -3246,14 +3505,22 @@
       <c r="W7" s="32" t="n"/>
       <c r="X7" s="32" t="n"/>
       <c r="Y7" s="33" t="n"/>
-      <c r="Z7" s="31" t="inlineStr">
+      <c r="Z7" s="27" t="inlineStr">
+        <is>
+          <t>Journal club</t>
+        </is>
+      </c>
+      <c r="AA7" s="31" t="inlineStr">
         <is>
           <t>Dry lab: flow statistics in R. Poster: figure 1 draft</t>
         </is>
       </c>
-      <c r="AA7" s="32" t="n"/>
-      <c r="AB7" s="32" t="n"/>
-      <c r="AC7" s="33" t="n"/>
+      <c r="AB7" s="33" t="n"/>
+      <c r="AC7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AD7" s="37" t="inlineStr">
         <is>
           <t>P05 Harvest supernatants. P06 ELISA IL-6 and TNF. P07 Griess</t>
@@ -3268,8 +3535,12 @@
         </is>
       </c>
       <c r="AI7" s="32" t="n"/>
-      <c r="AJ7" s="32" t="n"/>
-      <c r="AK7" s="33" t="n"/>
+      <c r="AJ7" s="33" t="n"/>
+      <c r="AK7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AL7" s="37" t="inlineStr">
         <is>
           <t>Plate reader runs, repeats where needed, clean-up. Check your own-vial culture</t>
@@ -3296,8 +3567,12 @@
         </is>
       </c>
       <c r="C8" s="32" t="n"/>
-      <c r="D8" s="32" t="n"/>
-      <c r="E8" s="33" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F8" s="37" t="inlineStr">
         <is>
           <t>P01 Thaw your own vial (viability = Exp 1 readout). P02 Seed Exp 2 plates from the staff culture</t>
@@ -3306,30 +3581,46 @@
       <c r="G8" s="32" t="n"/>
       <c r="H8" s="32" t="n"/>
       <c r="I8" s="33" t="n"/>
-      <c r="J8" s="31" t="inlineStr">
+      <c r="J8" s="27" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="K8" s="31" t="inlineStr">
         <is>
           <t>Dry lab: scRNA-seq part 3, score the tissue macrophages. Poster: methods</t>
         </is>
       </c>
-      <c r="K8" s="32" t="n"/>
-      <c r="L8" s="32" t="n"/>
-      <c r="M8" s="33" t="n"/>
+      <c r="L8" s="33" t="n"/>
+      <c r="M8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N8" s="37" t="inlineStr">
         <is>
           <t>P04 Polarize: M(-), M(IFNg), M(IL-4), M(IFNg+LPS), 24 h</t>
         </is>
       </c>
       <c r="O8" s="32" t="n"/>
-      <c r="P8" s="32" t="n"/>
-      <c r="Q8" s="33" t="n"/>
+      <c r="P8" s="33" t="n"/>
+      <c r="Q8" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
       <c r="R8" s="31" t="inlineStr">
         <is>
           <t>Dry lab: FlowJo gating of your own data, export statistics</t>
         </is>
       </c>
       <c r="S8" s="32" t="n"/>
-      <c r="T8" s="32" t="n"/>
-      <c r="U8" s="33" t="n"/>
+      <c r="T8" s="33" t="n"/>
+      <c r="U8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="V8" s="37" t="inlineStr">
         <is>
           <t>P04 Wash. P05 Challenge: LPS + your axis, 24 h. P08 Stain the unchallenged wells, acquire in the facility slot</t>
@@ -3338,14 +3629,22 @@
       <c r="W8" s="32" t="n"/>
       <c r="X8" s="32" t="n"/>
       <c r="Y8" s="33" t="n"/>
-      <c r="Z8" s="31" t="inlineStr">
+      <c r="Z8" s="27" t="inlineStr">
+        <is>
+          <t>Journal club</t>
+        </is>
+      </c>
+      <c r="AA8" s="31" t="inlineStr">
         <is>
           <t>Dry lab: flow statistics in R. Poster: figure 1 draft</t>
         </is>
       </c>
-      <c r="AA8" s="32" t="n"/>
-      <c r="AB8" s="32" t="n"/>
-      <c r="AC8" s="33" t="n"/>
+      <c r="AB8" s="33" t="n"/>
+      <c r="AC8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AD8" s="37" t="inlineStr">
         <is>
           <t>P05 Harvest supernatants. P06 ELISA IL-6 and TNF. P07 Griess</t>
@@ -3360,8 +3659,12 @@
         </is>
       </c>
       <c r="AI8" s="32" t="n"/>
-      <c r="AJ8" s="32" t="n"/>
-      <c r="AK8" s="33" t="n"/>
+      <c r="AJ8" s="33" t="n"/>
+      <c r="AK8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AL8" s="37" t="inlineStr">
         <is>
           <t>Plate reader runs, repeats where needed, clean-up. Check your own-vial culture</t>
@@ -3388,8 +3691,12 @@
         </is>
       </c>
       <c r="C9" s="32" t="n"/>
-      <c r="D9" s="32" t="n"/>
-      <c r="E9" s="33" t="n"/>
+      <c r="D9" s="33" t="n"/>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F9" s="31" t="inlineStr">
         <is>
           <t>Dry lab: scRNA-seq part 2, derive M(IFNg+LPS) and M(IL-4) signatures from the bulk RAW 264.7 dataset</t>
@@ -3398,22 +3705,34 @@
       <c r="G9" s="32" t="n"/>
       <c r="H9" s="32" t="n"/>
       <c r="I9" s="33" t="n"/>
-      <c r="J9" s="37" t="inlineStr">
+      <c r="J9" s="27" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="K9" s="37" t="inlineStr">
         <is>
           <t>P04 Polarize: M(-), M(IFNg), M(IL-4), M(IFNg+LPS), 24 h</t>
         </is>
       </c>
-      <c r="K9" s="32" t="n"/>
-      <c r="L9" s="32" t="n"/>
-      <c r="M9" s="33" t="n"/>
+      <c r="L9" s="33" t="n"/>
+      <c r="M9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N9" s="31" t="inlineStr">
         <is>
           <t>Dry lab: scRNA-seq part 3, score the tissue macrophages. Poster: methods</t>
         </is>
       </c>
       <c r="O9" s="32" t="n"/>
-      <c r="P9" s="32" t="n"/>
-      <c r="Q9" s="33" t="n"/>
+      <c r="P9" s="33" t="n"/>
+      <c r="Q9" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
       <c r="R9" s="37" t="inlineStr">
         <is>
           <t>P04 Wash. P05 Challenge: LPS + your axis, 24 h. P08 Stain the unchallenged wells, acquire in the facility slot</t>
@@ -3430,14 +3749,22 @@
       <c r="W9" s="32" t="n"/>
       <c r="X9" s="32" t="n"/>
       <c r="Y9" s="33" t="n"/>
-      <c r="Z9" s="37" t="inlineStr">
+      <c r="Z9" s="27" t="inlineStr">
+        <is>
+          <t>Journal club</t>
+        </is>
+      </c>
+      <c r="AA9" s="37" t="inlineStr">
         <is>
           <t>P05 Harvest supernatants. P06 ELISA IL-6 and TNF. P07 Griess</t>
         </is>
       </c>
-      <c r="AA9" s="32" t="n"/>
-      <c r="AB9" s="32" t="n"/>
-      <c r="AC9" s="33" t="n"/>
+      <c r="AB9" s="33" t="n"/>
+      <c r="AC9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AD9" s="31" t="inlineStr">
         <is>
           <t>Dry lab: flow statistics in R. Poster: figure 1 draft</t>
@@ -3452,8 +3779,12 @@
         </is>
       </c>
       <c r="AI9" s="32" t="n"/>
-      <c r="AJ9" s="32" t="n"/>
-      <c r="AK9" s="33" t="n"/>
+      <c r="AJ9" s="33" t="n"/>
+      <c r="AK9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AL9" s="31" t="inlineStr">
         <is>
           <t>Dry lab: ELISA and Griess analysis. Poster: results so far</t>
@@ -3480,8 +3811,12 @@
         </is>
       </c>
       <c r="C10" s="32" t="n"/>
-      <c r="D10" s="32" t="n"/>
-      <c r="E10" s="33" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F10" s="31" t="inlineStr">
         <is>
           <t>Dry lab: scRNA-seq part 2, derive M(IFNg+LPS) and M(IL-4) signatures from the bulk RAW 264.7 dataset</t>
@@ -3490,22 +3825,34 @@
       <c r="G10" s="32" t="n"/>
       <c r="H10" s="32" t="n"/>
       <c r="I10" s="33" t="n"/>
-      <c r="J10" s="37" t="inlineStr">
+      <c r="J10" s="27" t="inlineStr">
+        <is>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="K10" s="37" t="inlineStr">
         <is>
           <t>P04 Polarize: M(-), M(IFNg), M(IL-4), M(IFNg+LPS), 24 h</t>
         </is>
       </c>
-      <c r="K10" s="32" t="n"/>
-      <c r="L10" s="32" t="n"/>
-      <c r="M10" s="33" t="n"/>
+      <c r="L10" s="33" t="n"/>
+      <c r="M10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N10" s="31" t="inlineStr">
         <is>
           <t>Dry lab: scRNA-seq part 3, score the tissue macrophages. Poster: methods</t>
         </is>
       </c>
       <c r="O10" s="32" t="n"/>
-      <c r="P10" s="32" t="n"/>
-      <c r="Q10" s="33" t="n"/>
+      <c r="P10" s="33" t="n"/>
+      <c r="Q10" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
       <c r="R10" s="37" t="inlineStr">
         <is>
           <t>P04 Wash. P05 Challenge: LPS + your axis, 24 h. P08 Stain the unchallenged wells, acquire in the facility slot</t>
@@ -3522,14 +3869,22 @@
       <c r="W10" s="32" t="n"/>
       <c r="X10" s="32" t="n"/>
       <c r="Y10" s="33" t="n"/>
-      <c r="Z10" s="37" t="inlineStr">
+      <c r="Z10" s="27" t="inlineStr">
+        <is>
+          <t>Journal club</t>
+        </is>
+      </c>
+      <c r="AA10" s="37" t="inlineStr">
         <is>
           <t>P05 Harvest supernatants. P06 ELISA IL-6 and TNF. P07 Griess</t>
         </is>
       </c>
-      <c r="AA10" s="32" t="n"/>
-      <c r="AB10" s="32" t="n"/>
-      <c r="AC10" s="33" t="n"/>
+      <c r="AB10" s="33" t="n"/>
+      <c r="AC10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AD10" s="31" t="inlineStr">
         <is>
           <t>Dry lab: flow statistics in R. Poster: figure 1 draft</t>
@@ -3544,8 +3899,12 @@
         </is>
       </c>
       <c r="AI10" s="32" t="n"/>
-      <c r="AJ10" s="32" t="n"/>
-      <c r="AK10" s="33" t="n"/>
+      <c r="AJ10" s="33" t="n"/>
+      <c r="AK10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="AL10" s="31" t="inlineStr">
         <is>
           <t>Dry lab: ELISA and Griess analysis. Poster: results so far</t>
@@ -3703,7 +4062,7 @@
       </c>
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>One 24 h challenge arm only; the 6 h RNA arm belongs to the qPCR extension X01. A group that starts a step in the morning harvests it the next morning; pairs stay fixed within the week.</t>
+          <t>One 24 h challenge arm only; the 6 h RNA arm belongs to the qPCR extension X01. A group that starts a step in the morning harvests it the next morning; pairs stay fixed within the week. Mondays 12:00-13:00: IMHS Lunch Seminar. Tuesdays: Cutting Edge Immunology Seminar runs 16:30-17:30. Wed: groups C+D keep their cytometer slot (11:00-13:00) and have lunch afterwards.</t>
         </is>
       </c>
       <c r="C13" s="32" t="n"/>
@@ -3748,76 +4107,76 @@
     </row>
   </sheetData>
   <mergeCells count="70">
-    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="AH3:AO3"/>
+    <mergeCell ref="AH12:AO12"/>
+    <mergeCell ref="AH10:AJ10"/>
+    <mergeCell ref="R11:Y11"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="AA7:AB7"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="R3:Y3"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="AH4:AJ4"/>
     <mergeCell ref="AL7:AN7"/>
-    <mergeCell ref="AH3:AO3"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="AL4:AO4"/>
+    <mergeCell ref="AD7:AG7"/>
+    <mergeCell ref="Z11:AG11"/>
+    <mergeCell ref="V7:Y7"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="A1:AO1"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="AD8:AG8"/>
+    <mergeCell ref="AL8:AN8"/>
+    <mergeCell ref="R10:U10"/>
+    <mergeCell ref="R12:Y12"/>
+    <mergeCell ref="AL10:AN10"/>
+    <mergeCell ref="V10:Y10"/>
+    <mergeCell ref="AL9:AN9"/>
+    <mergeCell ref="V9:Y9"/>
+    <mergeCell ref="K10:L10"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="B13:AO13"/>
     <mergeCell ref="F9:I9"/>
-    <mergeCell ref="B13:AO13"/>
-    <mergeCell ref="AH12:AO12"/>
-    <mergeCell ref="N9:Q9"/>
-    <mergeCell ref="R11:Y11"/>
-    <mergeCell ref="Z4:AC4"/>
-    <mergeCell ref="AL4:AO4"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="AD7:AG7"/>
-    <mergeCell ref="V7:Y7"/>
-    <mergeCell ref="Z11:AG11"/>
-    <mergeCell ref="Z10:AC10"/>
-    <mergeCell ref="AH7:AK7"/>
-    <mergeCell ref="B12:I12"/>
-    <mergeCell ref="R9:U9"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="K9:L9"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="AA9:AB9"/>
     <mergeCell ref="AD4:AG4"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="Z9:AC9"/>
-    <mergeCell ref="R8:U8"/>
     <mergeCell ref="B11:I11"/>
     <mergeCell ref="F4:I4"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="A1:AO1"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="Z3:AG3"/>
+    <mergeCell ref="Z12:AG12"/>
+    <mergeCell ref="AH7:AJ7"/>
+    <mergeCell ref="V8:Y8"/>
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="K8:L8"/>
+    <mergeCell ref="AD10:AG10"/>
+    <mergeCell ref="AH11:AO11"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="J12:Q12"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="AH9:AJ9"/>
+    <mergeCell ref="R9:U9"/>
     <mergeCell ref="AD9:AG9"/>
     <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="AD8:AG8"/>
-    <mergeCell ref="AL8:AN8"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="N7:Q7"/>
-    <mergeCell ref="R10:U10"/>
-    <mergeCell ref="Z3:AG3"/>
-    <mergeCell ref="J10:M10"/>
-    <mergeCell ref="R12:Y12"/>
-    <mergeCell ref="Z12:AG12"/>
-    <mergeCell ref="AL10:AN10"/>
-    <mergeCell ref="R4:U4"/>
-    <mergeCell ref="V8:Y8"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="J9:M9"/>
-    <mergeCell ref="AH8:AK8"/>
-    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="Z4:AB4"/>
     <mergeCell ref="V4:Y4"/>
     <mergeCell ref="J11:Q11"/>
-    <mergeCell ref="AH4:AK4"/>
-    <mergeCell ref="R7:U7"/>
-    <mergeCell ref="V10:Y10"/>
-    <mergeCell ref="R3:Y3"/>
-    <mergeCell ref="Z7:AC7"/>
-    <mergeCell ref="AD10:AG10"/>
-    <mergeCell ref="AL9:AN9"/>
-    <mergeCell ref="AH11:AO11"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="AH10:AK10"/>
+    <mergeCell ref="R8:T8"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="N7:P7"/>
     <mergeCell ref="A2:AO2"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="V9:Y9"/>
-    <mergeCell ref="N8:Q8"/>
-    <mergeCell ref="J12:Q12"/>
     <mergeCell ref="J3:Q3"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="J4:M4"/>
-    <mergeCell ref="AH9:AK9"/>
-    <mergeCell ref="Z8:AC8"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="N10:Q10"/>
+    <mergeCell ref="AH8:AJ8"/>
+    <mergeCell ref="R7:T7"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3878,7 +4237,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Week 4: extensions, writing, poster (Mon 12 - Fri 16 April 2027)</t>
+          <t>Week 4: extensions, poster, presentations (Mon 12 - Fri 16 April 2027)</t>
         </is>
       </c>
     </row>
@@ -3900,61 +4259,61 @@
           <t>Mon 12 Apr</t>
         </is>
       </c>
-      <c r="C3" s="25" t="n"/>
-      <c r="D3" s="25" t="n"/>
-      <c r="E3" s="25" t="n"/>
-      <c r="F3" s="25" t="n"/>
-      <c r="G3" s="25" t="n"/>
-      <c r="H3" s="25" t="n"/>
-      <c r="I3" s="25" t="n"/>
+      <c r="C3" s="32" t="n"/>
+      <c r="D3" s="32" t="n"/>
+      <c r="E3" s="32" t="n"/>
+      <c r="F3" s="32" t="n"/>
+      <c r="G3" s="32" t="n"/>
+      <c r="H3" s="32" t="n"/>
+      <c r="I3" s="33" t="n"/>
       <c r="J3" s="25" t="inlineStr">
         <is>
           <t>Tue 13 Apr</t>
         </is>
       </c>
-      <c r="K3" s="25" t="n"/>
-      <c r="L3" s="25" t="n"/>
-      <c r="M3" s="25" t="n"/>
-      <c r="N3" s="25" t="n"/>
-      <c r="O3" s="25" t="n"/>
-      <c r="P3" s="25" t="n"/>
-      <c r="Q3" s="25" t="n"/>
+      <c r="K3" s="32" t="n"/>
+      <c r="L3" s="32" t="n"/>
+      <c r="M3" s="32" t="n"/>
+      <c r="N3" s="32" t="n"/>
+      <c r="O3" s="32" t="n"/>
+      <c r="P3" s="32" t="n"/>
+      <c r="Q3" s="33" t="n"/>
       <c r="R3" s="25" t="inlineStr">
         <is>
           <t>Wed 14 Apr</t>
         </is>
       </c>
-      <c r="S3" s="25" t="n"/>
-      <c r="T3" s="25" t="n"/>
-      <c r="U3" s="25" t="n"/>
-      <c r="V3" s="25" t="n"/>
-      <c r="W3" s="25" t="n"/>
-      <c r="X3" s="25" t="n"/>
-      <c r="Y3" s="25" t="n"/>
+      <c r="S3" s="32" t="n"/>
+      <c r="T3" s="32" t="n"/>
+      <c r="U3" s="32" t="n"/>
+      <c r="V3" s="32" t="n"/>
+      <c r="W3" s="32" t="n"/>
+      <c r="X3" s="32" t="n"/>
+      <c r="Y3" s="33" t="n"/>
       <c r="Z3" s="25" t="inlineStr">
         <is>
           <t>Thu 15 Apr</t>
         </is>
       </c>
-      <c r="AA3" s="25" t="n"/>
-      <c r="AB3" s="25" t="n"/>
-      <c r="AC3" s="25" t="n"/>
-      <c r="AD3" s="25" t="n"/>
-      <c r="AE3" s="25" t="n"/>
-      <c r="AF3" s="25" t="n"/>
-      <c r="AG3" s="25" t="n"/>
+      <c r="AA3" s="32" t="n"/>
+      <c r="AB3" s="32" t="n"/>
+      <c r="AC3" s="32" t="n"/>
+      <c r="AD3" s="32" t="n"/>
+      <c r="AE3" s="32" t="n"/>
+      <c r="AF3" s="32" t="n"/>
+      <c r="AG3" s="33" t="n"/>
       <c r="AH3" s="25" t="inlineStr">
         <is>
           <t>Fri 16 Apr</t>
         </is>
       </c>
-      <c r="AI3" s="25" t="n"/>
-      <c r="AJ3" s="25" t="n"/>
-      <c r="AK3" s="25" t="n"/>
-      <c r="AL3" s="25" t="n"/>
-      <c r="AM3" s="25" t="n"/>
-      <c r="AN3" s="25" t="n"/>
-      <c r="AO3" s="25" t="n"/>
+      <c r="AI3" s="32" t="n"/>
+      <c r="AJ3" s="32" t="n"/>
+      <c r="AK3" s="32" t="n"/>
+      <c r="AL3" s="32" t="n"/>
+      <c r="AM3" s="32" t="n"/>
+      <c r="AN3" s="32" t="n"/>
+      <c r="AO3" s="33" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="25" t="inlineStr">
@@ -3964,84 +4323,104 @@
       </c>
       <c r="B4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="C4" s="25" t="n"/>
-      <c r="D4" s="25" t="n"/>
-      <c r="E4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="C4" s="32" t="n"/>
+      <c r="D4" s="33" t="n"/>
+      <c r="E4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="F4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="G4" s="25" t="n"/>
-      <c r="H4" s="25" t="n"/>
-      <c r="I4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="G4" s="32" t="n"/>
+      <c r="H4" s="32" t="n"/>
+      <c r="I4" s="33" t="n"/>
       <c r="J4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="K4" s="25" t="n"/>
-      <c r="L4" s="25" t="n"/>
-      <c r="M4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="K4" s="32" t="n"/>
+      <c r="L4" s="33" t="n"/>
+      <c r="M4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="N4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="O4" s="25" t="n"/>
-      <c r="P4" s="25" t="n"/>
-      <c r="Q4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="O4" s="32" t="n"/>
+      <c r="P4" s="32" t="n"/>
+      <c r="Q4" s="33" t="n"/>
       <c r="R4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="S4" s="25" t="n"/>
-      <c r="T4" s="25" t="n"/>
-      <c r="U4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="S4" s="32" t="n"/>
+      <c r="T4" s="33" t="n"/>
+      <c r="U4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="V4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="W4" s="25" t="n"/>
-      <c r="X4" s="25" t="n"/>
-      <c r="Y4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="W4" s="32" t="n"/>
+      <c r="X4" s="32" t="n"/>
+      <c r="Y4" s="33" t="n"/>
       <c r="Z4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="AA4" s="25" t="n"/>
-      <c r="AB4" s="25" t="n"/>
-      <c r="AC4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="AA4" s="32" t="n"/>
+      <c r="AB4" s="33" t="n"/>
+      <c r="AC4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="AD4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="AE4" s="25" t="n"/>
-      <c r="AF4" s="25" t="n"/>
-      <c r="AG4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="AE4" s="32" t="n"/>
+      <c r="AF4" s="32" t="n"/>
+      <c r="AG4" s="33" t="n"/>
       <c r="AH4" s="25" t="inlineStr">
         <is>
-          <t>Morning 08:30-12:30</t>
-        </is>
-      </c>
-      <c r="AI4" s="25" t="n"/>
-      <c r="AJ4" s="25" t="n"/>
-      <c r="AK4" s="25" t="n"/>
+          <t>Morning 09:00-12:00</t>
+        </is>
+      </c>
+      <c r="AI4" s="32" t="n"/>
+      <c r="AJ4" s="33" t="n"/>
+      <c r="AK4" s="25" t="inlineStr">
+        <is>
+          <t>Lunch 12:00-13:00</t>
+        </is>
+      </c>
       <c r="AL4" s="25" t="inlineStr">
         <is>
-          <t>Afternoon 13:30-17:30</t>
-        </is>
-      </c>
-      <c r="AM4" s="25" t="n"/>
-      <c r="AN4" s="25" t="n"/>
-      <c r="AO4" s="25" t="n"/>
+          <t>Afternoon 13:00-17:00</t>
+        </is>
+      </c>
+      <c r="AM4" s="32" t="n"/>
+      <c r="AN4" s="32" t="n"/>
+      <c r="AO4" s="33" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
@@ -4051,202 +4430,202 @@
       </c>
       <c r="B5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="C5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="D5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="E5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="G5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="H5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="I5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="J5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="K5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="L5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="M5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="N5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="O5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="P5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="Q5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="R5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="S5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="T5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="U5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="V5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="W5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="X5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="Y5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="Z5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="AA5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="AB5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="AC5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="AD5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="AE5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="AF5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="AG5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
       <c r="AH5" s="25" t="inlineStr">
         <is>
-          <t>08:30</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="AI5" s="25" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>10:00</t>
         </is>
       </c>
       <c r="AJ5" s="25" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="AK5" s="25" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="AL5" s="25" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="AM5" s="25" t="inlineStr">
         <is>
-          <t>14:30</t>
+          <t>14:00</t>
         </is>
       </c>
       <c r="AN5" s="25" t="inlineStr">
         <is>
-          <t>15:30</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="AO5" s="25" t="inlineStr">
         <is>
-          <t>16:30</t>
+          <t>16:00</t>
         </is>
       </c>
     </row>
@@ -4260,7 +4639,11 @@
       <c r="B6" s="17" t="n"/>
       <c r="C6" s="17" t="n"/>
       <c r="D6" s="17" t="n"/>
-      <c r="E6" s="17" t="n"/>
+      <c r="E6" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F6" s="17" t="n"/>
       <c r="G6" s="17" t="n"/>
       <c r="H6" s="17" t="n"/>
@@ -4268,59 +4651,63 @@
       <c r="J6" s="17" t="n"/>
       <c r="K6" s="17" t="n"/>
       <c r="L6" s="17" t="n"/>
-      <c r="M6" s="17" t="n"/>
+      <c r="M6" s="41" t="n"/>
       <c r="N6" s="17" t="n"/>
       <c r="O6" s="17" t="n"/>
       <c r="P6" s="17" t="n"/>
       <c r="Q6" s="27" t="inlineStr">
         <is>
-          <t>Student-organised event (evening, from 17:30)</t>
+          <t>Cutting Edge Immunology Seminar 16:30-17:30</t>
         </is>
       </c>
       <c r="R6" s="27" t="inlineStr">
         <is>
-          <t>Scientific writing day: from data to argument, poster structure, figure design, honest limits</t>
-        </is>
-      </c>
-      <c r="S6" s="30" t="n"/>
-      <c r="T6" s="30" t="n"/>
-      <c r="U6" s="28" t="n"/>
-      <c r="V6" s="17" t="n"/>
-      <c r="W6" s="17" t="n"/>
-      <c r="X6" s="27" t="inlineStr">
+          <t>Lecture: scientific writing, from data to argument, poster structure, figure design, honest limits</t>
+        </is>
+      </c>
+      <c r="S6" s="41" t="n"/>
+      <c r="T6" s="41" t="n"/>
+      <c r="U6" s="41" t="n"/>
+      <c r="V6" s="41" t="n"/>
+      <c r="W6" s="41" t="n"/>
+      <c r="X6" s="41" t="n"/>
+      <c r="Y6" s="27" t="inlineStr">
         <is>
           <t>Failure round: each group presents one thing that went wrong and what it taught them</t>
         </is>
       </c>
-      <c r="Y6" s="28" t="n"/>
-      <c r="Z6" s="17" t="n"/>
-      <c r="AA6" s="17" t="n"/>
-      <c r="AB6" s="17" t="n"/>
-      <c r="AC6" s="17" t="n"/>
-      <c r="AD6" s="17" t="n"/>
-      <c r="AE6" s="17" t="n"/>
-      <c r="AF6" s="27" t="inlineStr">
-        <is>
-          <t>Feedback round with the teaching staff. Nerd ladder closes 17:00</t>
-        </is>
-      </c>
+      <c r="Z6" s="41" t="n"/>
+      <c r="AA6" s="41" t="n"/>
+      <c r="AB6" s="41" t="n"/>
+      <c r="AC6" s="41" t="n"/>
+      <c r="AD6" s="41" t="n"/>
+      <c r="AE6" s="27" t="inlineStr">
+        <is>
+          <t>Recap and Q&amp;A: the course in one hour, then open questions with the teaching staff</t>
+        </is>
+      </c>
+      <c r="AF6" s="30" t="n"/>
       <c r="AG6" s="28" t="n"/>
-      <c r="AH6" s="27" t="inlineStr">
-        <is>
-          <t>Poster presentations and discussion</t>
-        </is>
-      </c>
-      <c r="AI6" s="30" t="n"/>
-      <c r="AJ6" s="30" t="n"/>
-      <c r="AK6" s="28" t="n"/>
+      <c r="AH6" s="41" t="n"/>
+      <c r="AI6" s="41" t="n"/>
+      <c r="AJ6" s="27" t="inlineStr">
+        <is>
+          <t>Feedback round with the teaching staff; course evaluation</t>
+        </is>
+      </c>
+      <c r="AK6" s="41" t="n"/>
       <c r="AL6" s="27" t="inlineStr">
         <is>
-          <t>Prize, course evaluation, lab clean-up</t>
+          <t>Poster presentations and discussion; prize</t>
         </is>
       </c>
       <c r="AM6" s="30" t="n"/>
-      <c r="AN6" s="30" t="n"/>
-      <c r="AO6" s="28" t="n"/>
+      <c r="AN6" s="28" t="n"/>
+      <c r="AO6" s="27" t="inlineStr">
+        <is>
+          <t>Apéro</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="78" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
@@ -4335,8 +4722,12 @@
         </is>
       </c>
       <c r="C7" s="32" t="n"/>
-      <c r="D7" s="32" t="n"/>
-      <c r="E7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
+      <c r="E7" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F7" s="31" t="inlineStr">
         <is>
           <t>Dry lab: analysis of Exp 2. Poster: figures</t>
@@ -4351,64 +4742,104 @@
         </is>
       </c>
       <c r="K7" s="32" t="n"/>
-      <c r="L7" s="32" t="n"/>
-      <c r="M7" s="33" t="n"/>
+      <c r="L7" s="33" t="n"/>
+      <c r="M7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N7" s="31" t="inlineStr">
         <is>
           <t>Dry lab: extension analysis. Poster: figures and legends</t>
         </is>
       </c>
       <c r="O7" s="32" t="n"/>
-      <c r="P7" s="32" t="n"/>
-      <c r="Q7" s="33" t="n"/>
+      <c r="P7" s="33" t="n"/>
+      <c r="Q7" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
       <c r="R7" s="27" t="inlineStr">
         <is>
-          <t>Writing day</t>
-        </is>
-      </c>
-      <c r="S7" s="30" t="n"/>
-      <c r="T7" s="30" t="n"/>
-      <c r="U7" s="28" t="n"/>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="S7" s="39" t="inlineStr">
+        <is>
+          <t>Poster production with your supervisor</t>
+        </is>
+      </c>
+      <c r="T7" s="33" t="n"/>
+      <c r="U7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="V7" s="39" t="inlineStr">
         <is>
-          <t>Drafting with your supervisor</t>
-        </is>
-      </c>
-      <c r="W7" s="33" t="n"/>
-      <c r="X7" s="27" t="inlineStr">
+          <t>Poster production with your supervisor</t>
+        </is>
+      </c>
+      <c r="W7" s="32" t="n"/>
+      <c r="X7" s="33" t="n"/>
+      <c r="Y7" s="27" t="inlineStr">
         <is>
           <t>Failure round</t>
         </is>
       </c>
-      <c r="Y7" s="28" t="n"/>
       <c r="Z7" s="39" t="inlineStr">
         <is>
-          <t>Poster production</t>
+          <t>Poster production, final figures and legends</t>
         </is>
       </c>
       <c r="AA7" s="32" t="n"/>
-      <c r="AB7" s="32" t="n"/>
-      <c r="AC7" s="32" t="n"/>
-      <c r="AD7" s="32" t="n"/>
-      <c r="AE7" s="33" t="n"/>
-      <c r="AF7" s="27" t="inlineStr">
+      <c r="AB7" s="33" t="n"/>
+      <c r="AC7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="AD7" s="39" t="inlineStr">
+        <is>
+          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch; nerd ladder closes</t>
+        </is>
+      </c>
+      <c r="AE7" s="27" t="inlineStr">
+        <is>
+          <t>Recap and Q&amp;A</t>
+        </is>
+      </c>
+      <c r="AF7" s="30" t="n"/>
+      <c r="AG7" s="28" t="n"/>
+      <c r="AH7" s="31" t="inlineStr">
+        <is>
+          <t>Lab clean-up; notebook and group branch finalised</t>
+        </is>
+      </c>
+      <c r="AI7" s="33" t="n"/>
+      <c r="AJ7" s="27" t="inlineStr">
         <is>
           <t>Feedback round</t>
         </is>
       </c>
-      <c r="AG7" s="28" t="n"/>
-      <c r="AH7" s="27" t="inlineStr">
-        <is>
-          <t>Presentations, prize, evaluation, clean-up</t>
-        </is>
-      </c>
-      <c r="AI7" s="30" t="n"/>
-      <c r="AJ7" s="30" t="n"/>
-      <c r="AK7" s="30" t="n"/>
-      <c r="AL7" s="30" t="n"/>
+      <c r="AK7" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="AL7" s="27" t="inlineStr">
+        <is>
+          <t>Poster presentations</t>
+        </is>
+      </c>
       <c r="AM7" s="30" t="n"/>
-      <c r="AN7" s="30" t="n"/>
-      <c r="AO7" s="28" t="n"/>
+      <c r="AN7" s="28" t="n"/>
+      <c r="AO7" s="27" t="inlineStr">
+        <is>
+          <t>Apéro</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="78" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
@@ -4423,8 +4854,12 @@
         </is>
       </c>
       <c r="C8" s="32" t="n"/>
-      <c r="D8" s="32" t="n"/>
-      <c r="E8" s="33" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F8" s="31" t="inlineStr">
         <is>
           <t>Dry lab: analysis of Exp 2. Poster: figures</t>
@@ -4439,64 +4874,104 @@
         </is>
       </c>
       <c r="K8" s="32" t="n"/>
-      <c r="L8" s="32" t="n"/>
-      <c r="M8" s="33" t="n"/>
+      <c r="L8" s="33" t="n"/>
+      <c r="M8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N8" s="31" t="inlineStr">
         <is>
           <t>Dry lab: extension analysis. Poster: figures and legends</t>
         </is>
       </c>
       <c r="O8" s="32" t="n"/>
-      <c r="P8" s="32" t="n"/>
-      <c r="Q8" s="33" t="n"/>
+      <c r="P8" s="33" t="n"/>
+      <c r="Q8" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
       <c r="R8" s="27" t="inlineStr">
         <is>
-          <t>Writing day</t>
-        </is>
-      </c>
-      <c r="S8" s="30" t="n"/>
-      <c r="T8" s="30" t="n"/>
-      <c r="U8" s="28" t="n"/>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="S8" s="39" t="inlineStr">
+        <is>
+          <t>Poster production with your supervisor</t>
+        </is>
+      </c>
+      <c r="T8" s="33" t="n"/>
+      <c r="U8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="V8" s="39" t="inlineStr">
         <is>
-          <t>Drafting with your supervisor</t>
-        </is>
-      </c>
-      <c r="W8" s="33" t="n"/>
-      <c r="X8" s="27" t="inlineStr">
+          <t>Poster production with your supervisor</t>
+        </is>
+      </c>
+      <c r="W8" s="32" t="n"/>
+      <c r="X8" s="33" t="n"/>
+      <c r="Y8" s="27" t="inlineStr">
         <is>
           <t>Failure round</t>
         </is>
       </c>
-      <c r="Y8" s="28" t="n"/>
       <c r="Z8" s="39" t="inlineStr">
         <is>
-          <t>Poster production</t>
+          <t>Poster production, final figures and legends</t>
         </is>
       </c>
       <c r="AA8" s="32" t="n"/>
-      <c r="AB8" s="32" t="n"/>
-      <c r="AC8" s="32" t="n"/>
-      <c r="AD8" s="32" t="n"/>
-      <c r="AE8" s="33" t="n"/>
-      <c r="AF8" s="27" t="inlineStr">
+      <c r="AB8" s="33" t="n"/>
+      <c r="AC8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="AD8" s="39" t="inlineStr">
+        <is>
+          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch; nerd ladder closes</t>
+        </is>
+      </c>
+      <c r="AE8" s="27" t="inlineStr">
+        <is>
+          <t>Recap and Q&amp;A</t>
+        </is>
+      </c>
+      <c r="AF8" s="30" t="n"/>
+      <c r="AG8" s="28" t="n"/>
+      <c r="AH8" s="31" t="inlineStr">
+        <is>
+          <t>Lab clean-up; notebook and group branch finalised</t>
+        </is>
+      </c>
+      <c r="AI8" s="33" t="n"/>
+      <c r="AJ8" s="27" t="inlineStr">
         <is>
           <t>Feedback round</t>
         </is>
       </c>
-      <c r="AG8" s="28" t="n"/>
-      <c r="AH8" s="27" t="inlineStr">
-        <is>
-          <t>Presentations, prize, evaluation, clean-up</t>
-        </is>
-      </c>
-      <c r="AI8" s="30" t="n"/>
-      <c r="AJ8" s="30" t="n"/>
-      <c r="AK8" s="30" t="n"/>
-      <c r="AL8" s="30" t="n"/>
+      <c r="AK8" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="AL8" s="27" t="inlineStr">
+        <is>
+          <t>Poster presentations</t>
+        </is>
+      </c>
       <c r="AM8" s="30" t="n"/>
-      <c r="AN8" s="30" t="n"/>
-      <c r="AO8" s="28" t="n"/>
+      <c r="AN8" s="28" t="n"/>
+      <c r="AO8" s="27" t="inlineStr">
+        <is>
+          <t>Apéro</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="78" customHeight="1">
       <c r="A9" s="26" t="inlineStr">
@@ -4511,8 +4986,12 @@
         </is>
       </c>
       <c r="C9" s="32" t="n"/>
-      <c r="D9" s="32" t="n"/>
-      <c r="E9" s="33" t="n"/>
+      <c r="D9" s="33" t="n"/>
+      <c r="E9" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F9" s="38" t="inlineStr">
         <is>
           <t>Extension of your choice, or rescue path for Exp 2 (see Legend)</t>
@@ -4527,64 +5006,104 @@
         </is>
       </c>
       <c r="K9" s="32" t="n"/>
-      <c r="L9" s="32" t="n"/>
-      <c r="M9" s="33" t="n"/>
+      <c r="L9" s="33" t="n"/>
+      <c r="M9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N9" s="38" t="inlineStr">
         <is>
           <t>Extension, continued</t>
         </is>
       </c>
       <c r="O9" s="32" t="n"/>
-      <c r="P9" s="32" t="n"/>
-      <c r="Q9" s="33" t="n"/>
+      <c r="P9" s="33" t="n"/>
+      <c r="Q9" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
       <c r="R9" s="27" t="inlineStr">
         <is>
-          <t>Writing day</t>
-        </is>
-      </c>
-      <c r="S9" s="30" t="n"/>
-      <c r="T9" s="30" t="n"/>
-      <c r="U9" s="28" t="n"/>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="S9" s="39" t="inlineStr">
+        <is>
+          <t>Poster production with your supervisor</t>
+        </is>
+      </c>
+      <c r="T9" s="33" t="n"/>
+      <c r="U9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="V9" s="39" t="inlineStr">
         <is>
-          <t>Drafting with your supervisor</t>
-        </is>
-      </c>
-      <c r="W9" s="33" t="n"/>
-      <c r="X9" s="27" t="inlineStr">
+          <t>Poster production with your supervisor</t>
+        </is>
+      </c>
+      <c r="W9" s="32" t="n"/>
+      <c r="X9" s="33" t="n"/>
+      <c r="Y9" s="27" t="inlineStr">
         <is>
           <t>Failure round</t>
         </is>
       </c>
-      <c r="Y9" s="28" t="n"/>
       <c r="Z9" s="39" t="inlineStr">
         <is>
-          <t>Poster production</t>
+          <t>Poster production, final figures and legends</t>
         </is>
       </c>
       <c r="AA9" s="32" t="n"/>
-      <c r="AB9" s="32" t="n"/>
-      <c r="AC9" s="32" t="n"/>
-      <c r="AD9" s="32" t="n"/>
-      <c r="AE9" s="33" t="n"/>
-      <c r="AF9" s="27" t="inlineStr">
+      <c r="AB9" s="33" t="n"/>
+      <c r="AC9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="AD9" s="39" t="inlineStr">
+        <is>
+          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch; nerd ladder closes</t>
+        </is>
+      </c>
+      <c r="AE9" s="27" t="inlineStr">
+        <is>
+          <t>Recap and Q&amp;A</t>
+        </is>
+      </c>
+      <c r="AF9" s="30" t="n"/>
+      <c r="AG9" s="28" t="n"/>
+      <c r="AH9" s="31" t="inlineStr">
+        <is>
+          <t>Lab clean-up; notebook and group branch finalised</t>
+        </is>
+      </c>
+      <c r="AI9" s="33" t="n"/>
+      <c r="AJ9" s="27" t="inlineStr">
         <is>
           <t>Feedback round</t>
         </is>
       </c>
-      <c r="AG9" s="28" t="n"/>
-      <c r="AH9" s="27" t="inlineStr">
-        <is>
-          <t>Presentations, prize, evaluation, clean-up</t>
-        </is>
-      </c>
-      <c r="AI9" s="30" t="n"/>
-      <c r="AJ9" s="30" t="n"/>
-      <c r="AK9" s="30" t="n"/>
-      <c r="AL9" s="30" t="n"/>
+      <c r="AK9" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="AL9" s="27" t="inlineStr">
+        <is>
+          <t>Poster presentations</t>
+        </is>
+      </c>
       <c r="AM9" s="30" t="n"/>
-      <c r="AN9" s="30" t="n"/>
-      <c r="AO9" s="28" t="n"/>
+      <c r="AN9" s="28" t="n"/>
+      <c r="AO9" s="27" t="inlineStr">
+        <is>
+          <t>Apéro</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="78" customHeight="1">
       <c r="A10" s="26" t="inlineStr">
@@ -4599,8 +5118,12 @@
         </is>
       </c>
       <c r="C10" s="32" t="n"/>
-      <c r="D10" s="32" t="n"/>
-      <c r="E10" s="33" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="27" t="inlineStr">
+        <is>
+          <t>IMHS Lunch Seminar</t>
+        </is>
+      </c>
       <c r="F10" s="38" t="inlineStr">
         <is>
           <t>Extension of your choice, or rescue path for Exp 2 (see Legend)</t>
@@ -4615,64 +5138,104 @@
         </is>
       </c>
       <c r="K10" s="32" t="n"/>
-      <c r="L10" s="32" t="n"/>
-      <c r="M10" s="33" t="n"/>
+      <c r="L10" s="33" t="n"/>
+      <c r="M10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="N10" s="38" t="inlineStr">
         <is>
           <t>Extension, continued</t>
         </is>
       </c>
       <c r="O10" s="32" t="n"/>
-      <c r="P10" s="32" t="n"/>
-      <c r="Q10" s="33" t="n"/>
+      <c r="P10" s="33" t="n"/>
+      <c r="Q10" s="27" t="inlineStr">
+        <is>
+          <t>Seminar</t>
+        </is>
+      </c>
       <c r="R10" s="27" t="inlineStr">
         <is>
-          <t>Writing day</t>
-        </is>
-      </c>
-      <c r="S10" s="30" t="n"/>
-      <c r="T10" s="30" t="n"/>
-      <c r="U10" s="28" t="n"/>
+          <t>Lecture</t>
+        </is>
+      </c>
+      <c r="S10" s="39" t="inlineStr">
+        <is>
+          <t>Poster production with your supervisor</t>
+        </is>
+      </c>
+      <c r="T10" s="33" t="n"/>
+      <c r="U10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
       <c r="V10" s="39" t="inlineStr">
         <is>
-          <t>Drafting with your supervisor</t>
-        </is>
-      </c>
-      <c r="W10" s="33" t="n"/>
-      <c r="X10" s="27" t="inlineStr">
+          <t>Poster production with your supervisor</t>
+        </is>
+      </c>
+      <c r="W10" s="32" t="n"/>
+      <c r="X10" s="33" t="n"/>
+      <c r="Y10" s="27" t="inlineStr">
         <is>
           <t>Failure round</t>
         </is>
       </c>
-      <c r="Y10" s="28" t="n"/>
       <c r="Z10" s="39" t="inlineStr">
         <is>
-          <t>Poster production</t>
+          <t>Poster production, final figures and legends</t>
         </is>
       </c>
       <c r="AA10" s="32" t="n"/>
-      <c r="AB10" s="32" t="n"/>
-      <c r="AC10" s="32" t="n"/>
-      <c r="AD10" s="32" t="n"/>
-      <c r="AE10" s="33" t="n"/>
-      <c r="AF10" s="27" t="inlineStr">
+      <c r="AB10" s="33" t="n"/>
+      <c r="AC10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="AD10" s="39" t="inlineStr">
+        <is>
+          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch; nerd ladder closes</t>
+        </is>
+      </c>
+      <c r="AE10" s="27" t="inlineStr">
+        <is>
+          <t>Recap and Q&amp;A</t>
+        </is>
+      </c>
+      <c r="AF10" s="30" t="n"/>
+      <c r="AG10" s="28" t="n"/>
+      <c r="AH10" s="31" t="inlineStr">
+        <is>
+          <t>Lab clean-up; notebook and group branch finalised</t>
+        </is>
+      </c>
+      <c r="AI10" s="33" t="n"/>
+      <c r="AJ10" s="27" t="inlineStr">
         <is>
           <t>Feedback round</t>
         </is>
       </c>
-      <c r="AG10" s="28" t="n"/>
-      <c r="AH10" s="27" t="inlineStr">
-        <is>
-          <t>Presentations, prize, evaluation, clean-up</t>
-        </is>
-      </c>
-      <c r="AI10" s="30" t="n"/>
-      <c r="AJ10" s="30" t="n"/>
-      <c r="AK10" s="30" t="n"/>
-      <c r="AL10" s="30" t="n"/>
+      <c r="AK10" s="42" t="inlineStr">
+        <is>
+          <t>Lunch</t>
+        </is>
+      </c>
+      <c r="AL10" s="27" t="inlineStr">
+        <is>
+          <t>Poster presentations</t>
+        </is>
+      </c>
       <c r="AM10" s="30" t="n"/>
-      <c r="AN10" s="30" t="n"/>
-      <c r="AO10" s="28" t="n"/>
+      <c r="AN10" s="28" t="n"/>
+      <c r="AO10" s="27" t="inlineStr">
+        <is>
+          <t>Apéro</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="48" customHeight="1">
       <c r="A11" s="26" t="inlineStr">
@@ -4695,7 +5258,7 @@
       <c r="I11" s="33" t="n"/>
       <c r="J11" s="34" t="inlineStr">
         <is>
-          <t>Event logistics with the organisers. Rescue plates: challenge Tue.</t>
+          <t>Rescue plates: challenge Tue.</t>
         </is>
       </c>
       <c r="K11" s="32" t="n"/>
@@ -4707,7 +5270,7 @@
       <c r="Q11" s="33" t="n"/>
       <c r="R11" s="34" t="inlineStr">
         <is>
-          <t>Poster template distributed, printing booked [TODO]. Rescue plates: harvest 08:30.</t>
+          <t>Poster template distributed, printing booked [TODO: printer]. Rescue plates: harvest 09:00.</t>
         </is>
       </c>
       <c r="S11" s="32" t="n"/>
@@ -4719,7 +5282,7 @@
       <c r="Y11" s="33" t="n"/>
       <c r="Z11" s="34" t="inlineStr">
         <is>
-          <t>Printing. Rescue groups: ELISA in the morning, result on the poster by 17:00.</t>
+          <t>Posters printed Thu after 14:00 [TODO: printer]. Rescue groups: ELISA in the morning, result on the poster by 14:00.</t>
         </is>
       </c>
       <c r="AA11" s="32" t="n"/>
@@ -4731,7 +5294,7 @@
       <c r="AG11" s="33" t="n"/>
       <c r="AH11" s="34" t="inlineStr">
         <is>
-          <t>Jury, prize, evaluation form, clean-up checklist.</t>
+          <t>Jury, prize, evaluation form, clean-up checklist. Apéro ordered [TODO: catering].</t>
         </is>
       </c>
       <c r="AI11" s="32" t="n"/>
@@ -4771,7 +5334,7 @@
       <c r="Q12" s="33" t="n"/>
       <c r="R12" s="34" t="inlineStr">
         <is>
-          <t>Seminar room Wed to Fri. Printer [TODO]. Poster boards.</t>
+          <t>Seminar room Wed to Fri. Printer [TODO]. Poster boards. Apéro room [TODO: catering].</t>
         </is>
       </c>
       <c r="S12" s="32" t="n"/>
@@ -4806,7 +5369,7 @@
       </c>
       <c r="B13" s="34" t="inlineStr">
         <is>
-          <t>A full repeat of Exp 2 does not fit in week 4. Rescue path for a failed Exp 2: staff seed plates Fri 9 Apr, group polarizes Mon, challenges Tue, harvests Wed 08:30, ELISA Thu morning.</t>
+          <t>A full repeat of Exp 2 does not fit in week 4. Rescue path for a failed Exp 2: staff seed plates Fri 9 Apr, group polarizes Mon, challenges Tue, harvests Wed 09:00, ELISA Thu morning. Printing deadline Thu 14:00. Mondays 12:00-13:00: IMHS Lunch Seminar. Tuesdays: Cutting Edge Immunology Seminar runs 16:30-17:30.</t>
         </is>
       </c>
       <c r="C13" s="32" t="n"/>
@@ -4850,77 +5413,74 @@
       <c r="AO13" s="33" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="70">
-    <mergeCell ref="Z7:AE7"/>
-    <mergeCell ref="B9:E9"/>
+  <mergeCells count="67">
+    <mergeCell ref="V10:X10"/>
+    <mergeCell ref="AH3:AO3"/>
+    <mergeCell ref="R11:Y11"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="S10:T10"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="R3:Y3"/>
+    <mergeCell ref="S9:T9"/>
+    <mergeCell ref="AL6:AN6"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="AH4:AJ4"/>
+    <mergeCell ref="Z7:AB7"/>
+    <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="AL4:AO4"/>
+    <mergeCell ref="Z11:AG11"/>
+    <mergeCell ref="N8:P8"/>
+    <mergeCell ref="Z8:AB8"/>
+    <mergeCell ref="AH8:AI8"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="N10:P10"/>
+    <mergeCell ref="A1:AO1"/>
+    <mergeCell ref="B9:D9"/>
+    <mergeCell ref="AL8:AN8"/>
+    <mergeCell ref="AH10:AI10"/>
+    <mergeCell ref="AE6:AG6"/>
+    <mergeCell ref="AH9:AI9"/>
+    <mergeCell ref="AL10:AN10"/>
+    <mergeCell ref="Z9:AB9"/>
+    <mergeCell ref="AL9:AN9"/>
+    <mergeCell ref="AE7:AG7"/>
     <mergeCell ref="B13:AO13"/>
-    <mergeCell ref="AH3:AO3"/>
     <mergeCell ref="F9:I9"/>
-    <mergeCell ref="N9:Q9"/>
-    <mergeCell ref="R11:Y11"/>
-    <mergeCell ref="Z4:AC4"/>
-    <mergeCell ref="AL4:AO4"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="Z11:AG11"/>
-    <mergeCell ref="V8:W8"/>
-    <mergeCell ref="X8:Y8"/>
-    <mergeCell ref="Z8:AE8"/>
-    <mergeCell ref="X7:Y7"/>
-    <mergeCell ref="R9:U9"/>
+    <mergeCell ref="J4:L4"/>
     <mergeCell ref="AD4:AG4"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="AH8:AO8"/>
-    <mergeCell ref="R8:U8"/>
-    <mergeCell ref="V10:W10"/>
+    <mergeCell ref="R12:AO12"/>
     <mergeCell ref="B11:I11"/>
     <mergeCell ref="F4:I4"/>
-    <mergeCell ref="J8:M8"/>
-    <mergeCell ref="A1:AO1"/>
-    <mergeCell ref="R12:AO12"/>
+    <mergeCell ref="AE9:AG9"/>
+    <mergeCell ref="F10:I10"/>
+    <mergeCell ref="V7:X7"/>
+    <mergeCell ref="Z3:AG3"/>
+    <mergeCell ref="Z10:AB10"/>
+    <mergeCell ref="F7:I7"/>
+    <mergeCell ref="J8:L8"/>
+    <mergeCell ref="AH11:AO11"/>
+    <mergeCell ref="J10:L10"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="V9:X9"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="AE8:AG8"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="AE10:AG10"/>
     <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="AF10:AG10"/>
-    <mergeCell ref="B7:E7"/>
-    <mergeCell ref="AF6:AG6"/>
-    <mergeCell ref="AH10:AO10"/>
-    <mergeCell ref="V9:W9"/>
-    <mergeCell ref="F10:I10"/>
-    <mergeCell ref="N7:Q7"/>
-    <mergeCell ref="X9:Y9"/>
-    <mergeCell ref="R10:U10"/>
-    <mergeCell ref="AL6:AO6"/>
-    <mergeCell ref="Z3:AG3"/>
-    <mergeCell ref="J10:M10"/>
-    <mergeCell ref="AF9:AG9"/>
-    <mergeCell ref="Z10:AE10"/>
-    <mergeCell ref="AH9:AO9"/>
-    <mergeCell ref="R4:U4"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="J9:M9"/>
+    <mergeCell ref="Z4:AB4"/>
     <mergeCell ref="V4:Y4"/>
     <mergeCell ref="J11:Q11"/>
-    <mergeCell ref="AH4:AK4"/>
-    <mergeCell ref="R7:U7"/>
-    <mergeCell ref="Z9:AE9"/>
     <mergeCell ref="B12:Q12"/>
-    <mergeCell ref="R3:Y3"/>
-    <mergeCell ref="R6:U6"/>
-    <mergeCell ref="AH11:AO11"/>
-    <mergeCell ref="J7:M7"/>
-    <mergeCell ref="AF8:AG8"/>
-    <mergeCell ref="V7:W7"/>
+    <mergeCell ref="B7:D7"/>
     <mergeCell ref="A2:AO2"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="N8:Q8"/>
-    <mergeCell ref="X10:Y10"/>
-    <mergeCell ref="AF7:AG7"/>
+    <mergeCell ref="N7:P7"/>
     <mergeCell ref="J3:Q3"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="J4:M4"/>
-    <mergeCell ref="AH7:AO7"/>
-    <mergeCell ref="AH6:AK6"/>
-    <mergeCell ref="B10:E10"/>
-    <mergeCell ref="N10:Q10"/>
+    <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="V8:X8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Nerd factor instead of nerd ladder: drop points, scoring rules and prize mechanics
Section 6 becomes a menu of optional experiments and extensions; how they
are recognised is an open item. Failure round and assessment lose the
points language; the Gantt loses 'nerd ladder closes' and the legend says
nerd factor.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -869,7 +869,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Extension / nerd ladder (group's choice)</t>
+          <t>Extension / nerd factor (group's choice)</t>
         </is>
       </c>
     </row>
@@ -2848,59 +2848,59 @@
   </sheetData>
   <mergeCells count="55">
     <mergeCell ref="A1:AG1"/>
+    <mergeCell ref="AD10:AF10"/>
     <mergeCell ref="F9:I9"/>
+    <mergeCell ref="B8:D8"/>
     <mergeCell ref="R11:Y11"/>
     <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="Z11:AG11"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="V7:Y7"/>
     <mergeCell ref="J4:L4"/>
+    <mergeCell ref="N8:P8"/>
     <mergeCell ref="AA9:AB9"/>
+    <mergeCell ref="B12:I12"/>
+    <mergeCell ref="B10:D10"/>
+    <mergeCell ref="J7:L7"/>
+    <mergeCell ref="S8:T8"/>
     <mergeCell ref="AD4:AG4"/>
     <mergeCell ref="B11:I11"/>
     <mergeCell ref="S7:T7"/>
+    <mergeCell ref="N10:P10"/>
     <mergeCell ref="F4:I4"/>
+    <mergeCell ref="A2:AG2"/>
+    <mergeCell ref="N4:Q4"/>
+    <mergeCell ref="B9:D9"/>
     <mergeCell ref="N9:P9"/>
+    <mergeCell ref="Z4:AB4"/>
     <mergeCell ref="F10:I10"/>
+    <mergeCell ref="AD7:AF7"/>
     <mergeCell ref="Z3:AG3"/>
+    <mergeCell ref="R12:Y12"/>
     <mergeCell ref="Z12:AG12"/>
     <mergeCell ref="AA7:AB7"/>
     <mergeCell ref="V8:Y8"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="S10:T10"/>
+    <mergeCell ref="V4:Y4"/>
     <mergeCell ref="B4:D4"/>
+    <mergeCell ref="J11:Q11"/>
     <mergeCell ref="AD9:AF9"/>
     <mergeCell ref="J8:L8"/>
+    <mergeCell ref="B13:AG13"/>
     <mergeCell ref="R3:Y3"/>
+    <mergeCell ref="V10:Y10"/>
     <mergeCell ref="S9:T9"/>
     <mergeCell ref="AD8:AF8"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="N7:P7"/>
+    <mergeCell ref="V9:Y9"/>
     <mergeCell ref="J12:Q12"/>
     <mergeCell ref="J10:L10"/>
     <mergeCell ref="F8:I8"/>
+    <mergeCell ref="J3:Q3"/>
     <mergeCell ref="R4:T4"/>
     <mergeCell ref="J9:L9"/>
-    <mergeCell ref="AD10:AF10"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="Z11:AG11"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="V7:Y7"/>
-    <mergeCell ref="N8:P8"/>
-    <mergeCell ref="B12:I12"/>
-    <mergeCell ref="B10:D10"/>
-    <mergeCell ref="J7:L7"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="N10:P10"/>
-    <mergeCell ref="A2:AG2"/>
-    <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="B9:D9"/>
-    <mergeCell ref="Z4:AB4"/>
-    <mergeCell ref="AD7:AF7"/>
-    <mergeCell ref="R12:Y12"/>
-    <mergeCell ref="V4:Y4"/>
-    <mergeCell ref="J11:Q11"/>
-    <mergeCell ref="B13:AG13"/>
-    <mergeCell ref="V10:Y10"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="N7:P7"/>
-    <mergeCell ref="V9:Y9"/>
-    <mergeCell ref="J3:Q3"/>
     <mergeCell ref="AA8:AB8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4107,76 +4107,76 @@
     </row>
   </sheetData>
   <mergeCells count="70">
+    <mergeCell ref="B13:AO13"/>
+    <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="F9:I9"/>
     <mergeCell ref="AH3:AO3"/>
+    <mergeCell ref="AH10:AJ10"/>
     <mergeCell ref="AH12:AO12"/>
-    <mergeCell ref="AH10:AJ10"/>
     <mergeCell ref="R11:Y11"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="X6:Y6"/>
-    <mergeCell ref="AA7:AB7"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="R3:Y3"/>
-    <mergeCell ref="R4:T4"/>
-    <mergeCell ref="AH4:AJ4"/>
-    <mergeCell ref="AL7:AN7"/>
     <mergeCell ref="B8:D8"/>
+    <mergeCell ref="AA10:AB10"/>
+    <mergeCell ref="K9:L9"/>
     <mergeCell ref="AL4:AO4"/>
     <mergeCell ref="AD7:AG7"/>
     <mergeCell ref="Z11:AG11"/>
     <mergeCell ref="V7:Y7"/>
     <mergeCell ref="N8:P8"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="B3:I3"/>
+    <mergeCell ref="AH9:AJ9"/>
+    <mergeCell ref="AA9:AB9"/>
     <mergeCell ref="B12:I12"/>
     <mergeCell ref="B10:D10"/>
+    <mergeCell ref="R9:U9"/>
+    <mergeCell ref="AD4:AG4"/>
     <mergeCell ref="N10:P10"/>
+    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="AD9:AG9"/>
     <mergeCell ref="A1:AO1"/>
+    <mergeCell ref="N4:Q4"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="AD8:AG8"/>
+    <mergeCell ref="N9:P9"/>
     <mergeCell ref="AL8:AN8"/>
+    <mergeCell ref="Z4:AB4"/>
+    <mergeCell ref="F10:I10"/>
     <mergeCell ref="R10:U10"/>
     <mergeCell ref="R12:Y12"/>
-    <mergeCell ref="AL10:AN10"/>
-    <mergeCell ref="V10:Y10"/>
-    <mergeCell ref="AL9:AN9"/>
-    <mergeCell ref="V9:Y9"/>
-    <mergeCell ref="K10:L10"/>
-    <mergeCell ref="AA8:AB8"/>
-    <mergeCell ref="B13:AO13"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="AA10:AB10"/>
-    <mergeCell ref="K9:L9"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="AA9:AB9"/>
-    <mergeCell ref="AD4:AG4"/>
-    <mergeCell ref="B11:I11"/>
-    <mergeCell ref="F4:I4"/>
-    <mergeCell ref="F10:I10"/>
     <mergeCell ref="Z3:AG3"/>
     <mergeCell ref="Z12:AG12"/>
     <mergeCell ref="AH7:AJ7"/>
+    <mergeCell ref="AL10:AN10"/>
+    <mergeCell ref="X6:Y6"/>
+    <mergeCell ref="AA7:AB7"/>
     <mergeCell ref="V8:Y8"/>
     <mergeCell ref="F7:I7"/>
     <mergeCell ref="K8:L8"/>
+    <mergeCell ref="V4:Y4"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="J11:Q11"/>
+    <mergeCell ref="V10:Y10"/>
+    <mergeCell ref="R3:Y3"/>
+    <mergeCell ref="AL9:AN9"/>
     <mergeCell ref="AD10:AG10"/>
     <mergeCell ref="AH11:AO11"/>
-    <mergeCell ref="K7:L7"/>
-    <mergeCell ref="J12:Q12"/>
-    <mergeCell ref="F8:I8"/>
-    <mergeCell ref="T6:U6"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="AH9:AJ9"/>
-    <mergeCell ref="R9:U9"/>
-    <mergeCell ref="AD9:AG9"/>
-    <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="Z4:AB4"/>
-    <mergeCell ref="V4:Y4"/>
-    <mergeCell ref="J11:Q11"/>
     <mergeCell ref="R8:T8"/>
     <mergeCell ref="B7:D7"/>
     <mergeCell ref="N7:P7"/>
+    <mergeCell ref="K7:L7"/>
     <mergeCell ref="A2:AO2"/>
+    <mergeCell ref="V9:Y9"/>
+    <mergeCell ref="J12:Q12"/>
+    <mergeCell ref="F8:I8"/>
     <mergeCell ref="J3:Q3"/>
+    <mergeCell ref="T6:U6"/>
+    <mergeCell ref="R4:T4"/>
+    <mergeCell ref="K10:L10"/>
     <mergeCell ref="AH8:AJ8"/>
     <mergeCell ref="R7:T7"/>
+    <mergeCell ref="AA8:AB8"/>
+    <mergeCell ref="AH4:AJ4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="AD7" s="39" t="inlineStr">
         <is>
-          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch; nerd ladder closes</t>
+          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch</t>
         </is>
       </c>
       <c r="AE7" s="27" t="inlineStr">
@@ -4934,7 +4934,7 @@
       </c>
       <c r="AD8" s="39" t="inlineStr">
         <is>
-          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch; nerd ladder closes</t>
+          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch</t>
         </is>
       </c>
       <c r="AE8" s="27" t="inlineStr">
@@ -5066,7 +5066,7 @@
       </c>
       <c r="AD9" s="39" t="inlineStr">
         <is>
-          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch; nerd ladder closes</t>
+          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch</t>
         </is>
       </c>
       <c r="AE9" s="27" t="inlineStr">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="AD10" s="39" t="inlineStr">
         <is>
-          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch; nerd ladder closes</t>
+          <t>Final checks. Printing deadline 14:00: poster PDF committed to the group branch</t>
         </is>
       </c>
       <c r="AE10" s="27" t="inlineStr">
@@ -5415,72 +5415,72 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="V10:X10"/>
+    <mergeCell ref="B13:AO13"/>
+    <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="F9:I9"/>
     <mergeCell ref="AH3:AO3"/>
+    <mergeCell ref="B8:D8"/>
     <mergeCell ref="R11:Y11"/>
-    <mergeCell ref="S7:T7"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="S10:T10"/>
-    <mergeCell ref="B4:D4"/>
-    <mergeCell ref="R3:Y3"/>
-    <mergeCell ref="S9:T9"/>
-    <mergeCell ref="AL6:AN6"/>
-    <mergeCell ref="R4:T4"/>
-    <mergeCell ref="AH4:AJ4"/>
-    <mergeCell ref="Z7:AB7"/>
-    <mergeCell ref="AL7:AN7"/>
-    <mergeCell ref="B8:D8"/>
+    <mergeCell ref="V9:X9"/>
     <mergeCell ref="AL4:AO4"/>
     <mergeCell ref="Z11:AG11"/>
+    <mergeCell ref="B3:I3"/>
     <mergeCell ref="N8:P8"/>
+    <mergeCell ref="J4:L4"/>
+    <mergeCell ref="AE8:AG8"/>
+    <mergeCell ref="AH8:AI8"/>
     <mergeCell ref="Z8:AB8"/>
-    <mergeCell ref="AH8:AI8"/>
     <mergeCell ref="B10:D10"/>
     <mergeCell ref="J7:L7"/>
+    <mergeCell ref="S8:T8"/>
+    <mergeCell ref="AD4:AG4"/>
+    <mergeCell ref="R12:AO12"/>
     <mergeCell ref="N10:P10"/>
+    <mergeCell ref="S7:T7"/>
+    <mergeCell ref="B11:I11"/>
+    <mergeCell ref="F4:I4"/>
+    <mergeCell ref="AE10:AG10"/>
     <mergeCell ref="A1:AO1"/>
+    <mergeCell ref="N4:Q4"/>
     <mergeCell ref="B9:D9"/>
     <mergeCell ref="AL8:AN8"/>
+    <mergeCell ref="N9:P9"/>
     <mergeCell ref="AH10:AI10"/>
-    <mergeCell ref="AE6:AG6"/>
-    <mergeCell ref="AH9:AI9"/>
-    <mergeCell ref="AL10:AN10"/>
-    <mergeCell ref="Z9:AB9"/>
-    <mergeCell ref="AL9:AN9"/>
-    <mergeCell ref="AE7:AG7"/>
-    <mergeCell ref="B13:AO13"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="J4:L4"/>
-    <mergeCell ref="AD4:AG4"/>
-    <mergeCell ref="R12:AO12"/>
-    <mergeCell ref="B11:I11"/>
-    <mergeCell ref="F4:I4"/>
     <mergeCell ref="AE9:AG9"/>
+    <mergeCell ref="Z4:AB4"/>
     <mergeCell ref="F10:I10"/>
     <mergeCell ref="V7:X7"/>
+    <mergeCell ref="AE6:AG6"/>
     <mergeCell ref="Z3:AG3"/>
+    <mergeCell ref="AH9:AI9"/>
     <mergeCell ref="Z10:AB10"/>
+    <mergeCell ref="AL10:AN10"/>
+    <mergeCell ref="S10:T10"/>
     <mergeCell ref="F7:I7"/>
+    <mergeCell ref="V4:Y4"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="Z9:AB9"/>
+    <mergeCell ref="J11:Q11"/>
     <mergeCell ref="J8:L8"/>
+    <mergeCell ref="B12:Q12"/>
+    <mergeCell ref="Z7:AB7"/>
+    <mergeCell ref="R3:Y3"/>
+    <mergeCell ref="AL9:AN9"/>
+    <mergeCell ref="S9:T9"/>
     <mergeCell ref="AH11:AO11"/>
+    <mergeCell ref="B7:D7"/>
+    <mergeCell ref="AL6:AN6"/>
+    <mergeCell ref="AE7:AG7"/>
+    <mergeCell ref="A2:AO2"/>
+    <mergeCell ref="N7:P7"/>
     <mergeCell ref="J10:L10"/>
     <mergeCell ref="F8:I8"/>
-    <mergeCell ref="J9:L9"/>
-    <mergeCell ref="V9:X9"/>
-    <mergeCell ref="B3:I3"/>
-    <mergeCell ref="AE8:AG8"/>
-    <mergeCell ref="S8:T8"/>
-    <mergeCell ref="AE10:AG10"/>
-    <mergeCell ref="N4:Q4"/>
-    <mergeCell ref="Z4:AB4"/>
-    <mergeCell ref="V4:Y4"/>
-    <mergeCell ref="J11:Q11"/>
-    <mergeCell ref="B12:Q12"/>
-    <mergeCell ref="B7:D7"/>
-    <mergeCell ref="A2:AO2"/>
-    <mergeCell ref="N7:P7"/>
     <mergeCell ref="J3:Q3"/>
     <mergeCell ref="AH7:AI7"/>
+    <mergeCell ref="R4:T4"/>
     <mergeCell ref="V8:X8"/>
+    <mergeCell ref="J9:L9"/>
+    <mergeCell ref="AH4:AJ4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Merge schedule rework and nerd factor onto main; fix leftovers
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/schedule/Blockcourse_Gantt_FS2027.xlsx
+++ b/schedule/Blockcourse_Gantt_FS2027.xlsx
@@ -777,6 +777,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -885,6 +886,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="13" t="inlineStr">
         <is>
@@ -965,7 +967,7 @@
       </c>
       <c r="B20" s="14" t="inlineStr">
         <is>
-          <t>A full repeat of Exp 2 does not fit in week 4. A group whose Exp 2 failed takes the rescue path: staff seed plates Fri 9 April, polarize Mon 12, challenge Tue 13, harvest Wed 14 at 08:30, ELISA Thu 15 morning.</t>
+          <t>A full repeat of Exp 2 does not fit in week 4. A group whose Exp 2 failed takes the rescue path: staff seed plates Fri 9 April, polarize Mon 12, challenge Tue 13, harvest Wed 14 at 09:00, ELISA Thu 15 morning.</t>
         </is>
       </c>
     </row>
@@ -981,6 +983,7 @@
         </is>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
@@ -1073,6 +1076,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="16" t="inlineStr"/>
       <c r="B3" s="16" t="inlineStr">
@@ -1229,6 +1233,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
@@ -4107,10 +4112,10 @@
     </row>
   </sheetData>
   <mergeCells count="70">
+    <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="AH3:AO3"/>
+    <mergeCell ref="F9:I9"/>
     <mergeCell ref="B13:AO13"/>
-    <mergeCell ref="AL7:AN7"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="AH3:AO3"/>
     <mergeCell ref="AH10:AJ10"/>
     <mergeCell ref="AH12:AO12"/>
     <mergeCell ref="R11:Y11"/>
@@ -5415,10 +5420,10 @@
   </sheetData>
   <mergeCells count="67">
     <mergeCell ref="V10:X10"/>
+    <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="AH3:AO3"/>
+    <mergeCell ref="F9:I9"/>
     <mergeCell ref="B13:AO13"/>
-    <mergeCell ref="AL7:AN7"/>
-    <mergeCell ref="F9:I9"/>
-    <mergeCell ref="AH3:AO3"/>
     <mergeCell ref="B8:D8"/>
     <mergeCell ref="R11:Y11"/>
     <mergeCell ref="V9:X9"/>

</xml_diff>